<commit_message>
Update products from Google Sheets
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="produtcs" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="products" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +11,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="81">
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>brand</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>images</t>
+  </si>
+  <si>
+    <t>inStock</t>
+  </si>
+  <si>
+    <t>madeToOrder</t>
+  </si>
+  <si>
+    <t>color</t>
+  </si>
+  <si>
+    <t>sizes</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
   <si>
     <t>Футболка Dior</t>
   </si>
@@ -22,7 +61,7 @@
     <t>12000</t>
   </si>
   <si>
-    <t>RUB</t>
+    <t>₽</t>
   </si>
   <si>
     <t>Материал хлопок</t>
@@ -221,7 +260,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -232,6 +271,21 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FFE4E4E4"/>
+      <name val="Menlo"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FFE4E4E4"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
@@ -246,26 +300,49 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF9A9A9A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF9A9A9A"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF9A9A9A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF9A9A9A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -486,926 +563,967 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1">
-        <v>1.0</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="M1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>3</v>
+      <c r="E3" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>3</v>
+        <v>38</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>8</v>
+        <v>39</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>8</v>
+        <v>43</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>9.0</v>
+        <v>8.0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>8</v>
+        <v>47</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>3</v>
+        <v>49</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>8</v>
+        <v>51</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>3</v>
+        <v>53</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>8</v>
+        <v>56</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>3</v>
+        <v>53</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>8</v>
+        <v>60</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>3</v>
+        <v>53</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>8</v>
+        <v>62</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>14.0</v>
+        <v>13.0</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>3</v>
+        <v>64</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>8</v>
+        <v>65</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>8</v>
+        <v>66</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>3</v>
+        <v>71</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>18.0</v>
+        <v>17.0</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>3</v>
+        <v>64</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>8</v>
+        <v>74</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="G19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
         <v>20.0</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21" s="3"/>
+      <c r="B21" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="22">
-      <c r="E22" s="3"/>
+      <c r="E22" s="7"/>
     </row>
     <row r="23">
-      <c r="E23" s="3"/>
+      <c r="E23" s="7"/>
     </row>
     <row r="24">
-      <c r="E24" s="3"/>
+      <c r="E24" s="7"/>
     </row>
     <row r="25">
-      <c r="E25" s="3"/>
+      <c r="E25" s="7"/>
     </row>
     <row r="26">
-      <c r="E26" s="3"/>
+      <c r="E26" s="7"/>
     </row>
     <row r="27">
-      <c r="E27" s="3"/>
+      <c r="E27" s="7"/>
     </row>
     <row r="28">
-      <c r="E28" s="3"/>
+      <c r="E28" s="7"/>
     </row>
     <row r="29">
-      <c r="E29" s="3"/>
+      <c r="E29" s="7"/>
     </row>
     <row r="30">
-      <c r="E30" s="3"/>
+      <c r="E30" s="7"/>
     </row>
     <row r="31">
-      <c r="E31" s="3"/>
+      <c r="E31" s="7"/>
     </row>
     <row r="32">
-      <c r="E32" s="3"/>
+      <c r="E32" s="7"/>
     </row>
     <row r="33">
-      <c r="E33" s="3"/>
+      <c r="E33" s="7"/>
     </row>
     <row r="34">
-      <c r="E34" s="3"/>
+      <c r="E34" s="7"/>
     </row>
     <row r="35">
-      <c r="E35" s="3"/>
+      <c r="E35" s="7"/>
     </row>
     <row r="36">
-      <c r="E36" s="3"/>
+      <c r="E36" s="7"/>
     </row>
     <row r="37">
-      <c r="E37" s="3"/>
+      <c r="E37" s="7"/>
     </row>
     <row r="38">
-      <c r="E38" s="3"/>
+      <c r="E38" s="7"/>
     </row>
     <row r="39">
-      <c r="E39" s="3"/>
+      <c r="E39" s="7"/>
     </row>
     <row r="40">
-      <c r="E40" s="3"/>
+      <c r="E40" s="7"/>
     </row>
     <row r="41">
-      <c r="E41" s="3"/>
+      <c r="E41" s="7"/>
     </row>
     <row r="42">
-      <c r="E42" s="3"/>
+      <c r="E42" s="7"/>
     </row>
     <row r="43">
-      <c r="E43" s="3"/>
+      <c r="E43" s="7"/>
     </row>
     <row r="44">
-      <c r="E44" s="3"/>
+      <c r="E44" s="7"/>
     </row>
     <row r="45">
-      <c r="E45" s="3"/>
+      <c r="E45" s="7"/>
     </row>
     <row r="46">
-      <c r="E46" s="3"/>
+      <c r="E46" s="7"/>
     </row>
     <row r="47">
-      <c r="E47" s="3"/>
+      <c r="E47" s="7"/>
     </row>
     <row r="48">
-      <c r="E48" s="3"/>
+      <c r="E48" s="7"/>
     </row>
     <row r="49">
-      <c r="E49" s="3"/>
+      <c r="E49" s="7"/>
     </row>
     <row r="50">
-      <c r="E50" s="3"/>
+      <c r="E50" s="7"/>
     </row>
     <row r="51">
-      <c r="E51" s="3"/>
+      <c r="E51" s="7"/>
+    </row>
+    <row r="52">
+      <c r="E52" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="H1"/>
-    <hyperlink r:id="rId2" ref="H2"/>
-    <hyperlink r:id="rId3" ref="H3"/>
-    <hyperlink r:id="rId4" ref="H5"/>
-    <hyperlink r:id="rId5" ref="H16"/>
-    <hyperlink r:id="rId6" ref="H19"/>
+    <hyperlink r:id="rId1" ref="H2"/>
+    <hyperlink r:id="rId2" ref="H3"/>
+    <hyperlink r:id="rId3" ref="H4"/>
+    <hyperlink r:id="rId4" ref="H6"/>
+    <hyperlink r:id="rId5" ref="H17"/>
+    <hyperlink r:id="rId6" ref="H20"/>
   </hyperlinks>
   <drawing r:id="rId7"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplify product card overlays and update products.xlsx
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a/ЛСсайт/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{433046AA-9CD3-F148-A12D-67645EE98721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2D99DD-513E-7C48-BBEA-C430C895E7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="185">
   <si>
     <t>id</t>
   </si>
@@ -112,9 +112,6 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773656988/tg-products/nd2ndp0l7e13lpno5hpb.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657069/tg-products/bhgxysknyx1l2jk9u3rn.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657073/tg-products/kwpdv0osksg4zvrudyr0.jpg</t>
-  </si>
-  <si>
     <t>розовый</t>
   </si>
   <si>
@@ -139,9 +136,6 @@
     <t>Valentino</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657079/tg-products/z6chjwosq1tsmqmouhm6.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657082/tg-products/pw2oxr6l74zinnsgk6w0.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657085/tg-products/tjrhi6r2xvl4ygdssfrd.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657088/tg-products/d7dqmbr96bs05rswdldf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657095/tg-products/thgk4m3rmewg5utuvs7v.jpg</t>
-  </si>
-  <si>
     <t>голбой</t>
   </si>
   <si>
@@ -151,9 +145,6 @@
     <t>24000</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657098/tg-products/rsyptz7fwqfelmxy6ydw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657100/tg-products/m9mzf7z9totbgmrwy7ly.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657147/tg-products/xncdhbxhflitmubbgm9a.jpg</t>
-  </si>
-  <si>
     <t>голубой</t>
   </si>
   <si>
@@ -163,9 +154,6 @@
     <t>Материал кашемир</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657152/tg-products/jdsaqx31zr7cjvimmbxg.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657154/tg-products/fnys55hvcsadqrlc19hf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657157/tg-products/bxyru9eahuawsrqxoquo.jpg</t>
-  </si>
-  <si>
     <t>Футболка Louis Vuitton</t>
   </si>
   <si>
@@ -175,9 +163,6 @@
     <t>14000</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657159/tg-products/ucwhnnndkjvjj0rfgch7.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657161/tg-products/rxt1h8ofjx9eqvv2sqqz.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657164/tg-products/sswmebnlaxvoisvuawct.jpg</t>
-  </si>
-  <si>
     <t>Брюки Chanel</t>
   </si>
   <si>
@@ -190,9 +175,6 @@
     <t>Материал шелк и полиэстер</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657167/tg-products/j01zqhctwihp1juowjcy.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657170/tg-products/ev23h726ddf3tyt3rrae.jpg</t>
-  </si>
-  <si>
     <t>Рубашка Chanel</t>
   </si>
   <si>
@@ -202,36 +184,21 @@
     <t>Материал шелк</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657172/tg-products/wh9xzqswuvwgbmafmluz.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657174/tg-products/tze9yngyvqu8mnmasdvh.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657180/tg-products/m7pvci0iacztyp6pr3u7.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657182/tg-products/ommnvpvdo3yckyr5vbst.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657185/tg-products/bfsigfbw8ak8ka48onij.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657188/tg-products/l0gopq2c6musnlcfoz5z.jpg</t>
-  </si>
-  <si>
     <t>Топ Chanel</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657191/tg-products/ppvqbfgli5m1qmlkdpuw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657194/tg-products/a9mwskgzuxgao8coydke.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657197/tg-products/iq1cgfpw5bqfqcwfzyjq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657199/tg-products/oaexxi222us3u7dda6d0.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657202/tg-products/fvclhikjdln1hshxsis1.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657206/tg-products/soyqphkxylqiok1qp2ci.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657208/tg-products/bjdt7gfw682yhvobjcbh.jpg</t>
-  </si>
-  <si>
     <t>Футболка Celine</t>
   </si>
   <si>
     <t>Celine</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657211/tg-products/yfbejf19ousiedoa3ro8.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657213/tg-products/gdxmqamyyx5qlu7xkcjk.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657325/tg-products/lxnge5xudt6hxnblg5qt.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657328/tg-products/qs1va9md29sm0hkbimbu.jpg</t>
-  </si>
-  <si>
     <t>Топ Dior</t>
   </si>
   <si>
     <t>20000</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657330/tg-products/a5b9x9ksqrjahiqvzb2d.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657332/tg-products/iqzouoeual1vbxgmuiul.jpg</t>
-  </si>
-  <si>
     <t>Рубашка Prada</t>
   </si>
   <si>
@@ -244,12 +211,6 @@
     <t>Блузка Chloe</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657393/tg-products/jsaz5u3qrqttlngmnfgv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657423/tg-products/godbajmqrjcjbz8prrlc.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657426/tg-products/kpizlbff8kyvcowsrsqj.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657428/tg-products/bouempg5bkozzmhbe2xg.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657430/tg-products/u2nmfiipteo7m94vp7vw.jpg</t>
-  </si>
-  <si>
     <t>Шорты Miumiu</t>
   </si>
   <si>
@@ -262,9 +223,6 @@
     <t>Лонгслив Miumiu</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657434/tg-products/petjj0v2jgsvjhxu2t2y.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657436/tg-products/glwgfyzvoxrivzb8bvrc.jpg</t>
-  </si>
-  <si>
     <t>Cумка Bottega Veneta</t>
   </si>
   <si>
@@ -277,9 +235,6 @@
     <t>bags</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816112/tg-products/pitfg5ru3uln0ddtof3r.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816115/tg-products/lxtt0igpkxfq0wsizh7i.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816337/tg-products/phyafi9uw9fmj6bc1ci7.jpg</t>
-  </si>
-  <si>
     <t>зеленый</t>
   </si>
   <si>
@@ -295,9 +250,6 @@
     <t>Материал нейлон</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816339/tg-products/fsfrtxbtdfo0s02zgsmd.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816341/tg-products/jn9iloy9lyux1gyegmxx.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816513/tg-products/pakoq54nopsn1hndpde9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816516/tg-products/ayxvxbmsubumkq11iab2.jpg</t>
-  </si>
-  <si>
     <t>Поло Miumiu</t>
   </si>
   <si>
@@ -307,18 +259,9 @@
     <t>Лонгслив Celine</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816630/tg-products/rzhuphpv934hsspwjcac.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816632/tg-products/wcczjq0eafp70qnq7yxb.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816635/tg-products/y8abqxdgeqradf9v8kn3.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816898/tg-products/wc9dbqqabjssntstope5.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816901/tg-products/nqgnpv4nhjbwiu7hjvtq.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816903/tg-products/di8f3jkcpgga3r9qmcyb.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817251/tg-products/i734pcf89hwihtvndvkd.jpg</t>
-  </si>
-  <si>
     <t>Юбка Prada</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817254/tg-products/rizqedb0kzzpw8mad3b6.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817256/tg-products/d1fiiqkepfx7wueogmvt.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817313/tg-products/b7eg1yovz5ynm5blftej.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817315/tg-products/vcl3bibo013ehsgxzfpm.jpg</t>
-  </si>
-  <si>
     <t>Джинсы Brunello Cucinelli</t>
   </si>
   <si>
@@ -328,36 +271,21 @@
     <t>Материал Хлопок</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817318/tg-products/ylgzcd8hw89ryxuy9wgb.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817502/tg-products/yxbdwftwbt2nwhpdltis.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817505/tg-products/dbfkikayeksfittpg3c3.jpg</t>
-  </si>
-  <si>
     <t>Рубашка Valentino</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817508/tg-products/w1svjywfln1pih49hg8t.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817642/tg-products/lmdkaqnxyh5f14hohww3.jpg</t>
-  </si>
-  <si>
     <t>Майка Prada</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817645/tg-products/jnynyokfyhj3qsyx9xnj.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817647/tg-products/bfrmyir175yqnr9ob40p.jpg</t>
-  </si>
-  <si>
     <t>черный</t>
   </si>
   <si>
     <t>Рубашка Brunello Cucinelli</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817754/tg-products/cpfreiffmhgyzd93datj.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817756/tg-products/sf2k3vztxn4ic512gzsx.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817758/tg-products/jh8oydbviq4dukpfcnu8.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817777/tg-products/db51stpkjb9qyt1xf4oa.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817780/tg-products/riy5n5zhqnbwt4pmjth6.jpg</t>
-  </si>
-  <si>
     <t>коричневый</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817782/tg-products/ufiiywegloio1x0gqdup.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773830691/tg-products/dhjldil5xwzxwdvvsy4d.jpg</t>
-  </si>
-  <si>
     <t>Кроссовки Hermes</t>
   </si>
   <si>
@@ -367,9 +295,6 @@
     <t>shoes</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773830697/tg-products/t58uzuebmuahcobfnwve.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773830700/tg-products/rodsy5dk3l0a8xiqcril.jpg</t>
-  </si>
-  <si>
     <t>35 36 37 38 39 40</t>
   </si>
   <si>
@@ -481,60 +406,27 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833016/tg-products/jeoxdlgvx885ilu5ppjy.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833036/tg-products/fwfq56v1fhvye5vn7tca.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833663/tg-products/dqdejnonpwlysoyuulm5.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833667/tg-products/ajna4isso0n29hf2pece.jpg</t>
-  </si>
-  <si>
     <t>Сумка Bottega Veneta</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833670/tg-products/hwxadkpms9jh21fxw3jy.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833745/tg-products/p55aadptaigq65lca5gw.jpg</t>
-  </si>
-  <si>
     <t>39x25x18.5 см</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833753/tg-products/n1h2jljzzvnvbb5vuqm9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833757/tg-products/hlit3tg9hcvolmikvqj8.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833786/tg-products/itgmxlmrxnmqpluutqyg.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833789/tg-products/hjhf0t97cpv5ikiaachr.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833792/tg-products/i43cheic3jgchzlrutej.jpg</t>
-  </si>
-  <si>
     <t>бордовый</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833835/tg-products/ybmj3n0lwzafivnpl1uw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833838/tg-products/js8z3k0d0dfxtckeecxz.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833841/tg-products/ie7ieg44kpg7mqziwb5l.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833909/tg-products/k4pbk87mhwndsrpoz0js.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833913/tg-products/to7x83ks9mydmb4zwzfs.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833917/tg-products/a0zubiodyon2xd1rfik2.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833932/tg-products/fy8m8n6xt24oowu69bdl.jpg</t>
-  </si>
-  <si>
     <t>красный</t>
   </si>
   <si>
     <t>21x11x9 см</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833936/tg-products/kf5evug3y3afwlfsxe7k.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833938/tg-products/uqpacz5ywnypbmulzpad.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833962/tg-products/vxgzb3plkv0lljydi0ql.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833965/tg-products/wsn7tqksvlrvoj5odctx.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833969/tg-products/pboh9oo8jcgcnpj5bytv.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834028/tg-products/dll5ilxr2cvrfrmb5zr6.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834031/tg-products/tjayysex8bzeuofpthiq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834035/tg-products/isuda1chzxqhf49cazlb.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834086/tg-products/q4zbjv25kvxpeiurtwb7.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834089/tg-products/ah9ybpq58ps4c5cw1gsc.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834092/tg-products/uy6cqzf4y0uro9otz8hf.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834321/tg-products/k4bkfhn2f10ssvrtgm5u.jpg</t>
   </si>
   <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834325/tg-products/z3olimdqvrbbchauxyp8.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835308/tg-products/zyxgjrvtjv4ea5yd2whz.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835311/tg-products/nj42wapveufuq94tux7b.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835315/tg-products/ingo8tua2bmu4cjt7m9b.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835498/tg-products/ixvsxn6ng5h39sv1jhkl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835503/tg-products/uyhrzy2a1xgzdlghyspy.jpg</t>
-  </si>
-  <si>
     <t>17x10x6 см</t>
   </si>
   <si>
@@ -550,12 +442,6 @@
     <t>Куртка Brunello Cucinelli</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835561/tg-products/djmln37ynprbvnw9j3kf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835567/tg-products/bcloy4laepu7xjnximux.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835577/tg-products/ms4qzopjvfmnvxe4fyql.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835610/tg-products/ry6zindmjsnornscgrre.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835614/tg-products/maa475djsqbflpsu43uq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835617/tg-products/xfa7pbpame6l5jhjcy2r.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835622/tg-products/xpswgt46xryxgyiizb5q.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835759/tg-products/iwhcisnvkwzcfly0mlih.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835767/tg-products/btetnlvzi7jaytlrij2j.jpg</t>
-  </si>
-  <si>
     <t>Пиджак Loro Piana</t>
   </si>
   <si>
@@ -565,7 +451,130 @@
     <t>Материал шерсть</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835773/tg-products/eokilkgoajhxjgjaknxs.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835778/tg-products/auyz4azjhufbybxeoccy.jpg</t>
+    <t>52000</t>
+  </si>
+  <si>
+    <t>13000</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835773/tg-products/eokilkgoajhxjgjaknxs.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835778/tg-products/auyz4azjhufbybxeoccy.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835767/tg-products/btetnlvzi7jaytlrij2j.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835759/tg-products/iwhcisnvkwzcfly0mlih.jpg</t>
+  </si>
+  <si>
+    <t>Юбка Brunello Cucinelli</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835561/tg-products/djmln37ynprbvnw9j3kf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835567/tg-products/bcloy4laepu7xjnximux.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835622/tg-products/xpswgt46xryxgyiizb5q.jpg,  https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835577/tg-products/ms4qzopjvfmnvxe4fyql.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835610/tg-products/ry6zindmjsnornscgrre.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835614/tg-products/maa475djsqbflpsu43uq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835617/tg-products/xfa7pbpame6l5jhjcy2r.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833036/tg-products/fwfq56v1fhvye5vn7tca.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833670/tg-products/hwxadkpms9jh21fxw3jy.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833753/tg-products/n1h2jljzzvnvbb5vuqm9.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833789/tg-products/hjhf0t97cpv5ikiaachr.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833835/tg-products/ybmj3n0lwzafivnpl1uw.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833909/tg-products/k4pbk87mhwndsrpoz0js.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833936/tg-products/kf5evug3y3afwlfsxe7k.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833962/tg-products/vxgzb3plkv0lljydi0ql.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834086/tg-products/q4zbjv25kvxpeiurtwb7.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://res.cloudinary.com/dlexrnrhe/image/upload/v1773834028/tg-products/dll5ilxr2cvrfrmb5zr6.jpg </t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835308/tg-products/zyxgjrvtjv4ea5yd2whz.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773830697/tg-products/t58uzuebmuahcobfnwve.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817782/tg-products/ufiiywegloio1x0gqdup.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817754/tg-products/cpfreiffmhgyzd93datj.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817645/tg-products/jnynyokfyhj3qsyx9xnj.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817508/tg-products/w1svjywfln1pih49hg8t.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817318/tg-products/ylgzcd8hw89ryxuy9wgb.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816903/tg-products/di8f3jkcpgga3r9qmcyb.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://res.cloudinary.com/dlexrnrhe/image/upload/v1773817254/tg-products/rizqedb0kzzpw8mad3b6.jpg </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816630/tg-products/rzhuphpv934hsspwjcac.jpg </t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816339/tg-products/fsfrtxbtdfo0s02zgsmd.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657434/tg-products/petjj0v2jgsvjhxu2t2y.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773816112/tg-products/pitfg5ru3uln0ddtof3r.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657428/tg-products/bouempg5bkozzmhbe2xg.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657393/tg-products/jsaz5u3qrqttlngmnfgv.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657330/tg-products/a5b9x9ksqrjahiqvzb2d.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657325/tg-products/lxnge5xudt6hxnblg5qt.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657211/tg-products/yfbejf19ousiedoa3ro8.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657191/tg-products/ppvqbfgli5m1qmlkdpuw.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657172/tg-products/wh9xzqswuvwgbmafmluz.jpg,</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657167/tg-products/j01zqhctwihp1juowjcy.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657159/tg-products/ucwhnnndkjvjj0rfgch7.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657152/tg-products/jdsaqx31zr7cjvimmbxg.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657098/tg-products/rsyptz7fwqfelmxy6ydw.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657079/tg-products/z6chjwosq1tsmqmouhm6.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657069/tg-products/bhgxysknyx1l2jk9u3rn.jpg</t>
   </si>
 </sst>
 </file>
@@ -676,7 +685,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
@@ -689,6 +698,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -1101,17 +1111,17 @@
       <c r="G5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>23</v>
@@ -1125,34 +1135,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>23</v>
@@ -1166,10 +1176,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>15</v>
@@ -1183,8 +1193,8 @@
       <c r="G7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>39</v>
+      <c r="H7" s="11" t="s">
+        <v>183</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
@@ -1193,7 +1203,7 @@
         <v>21</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>23</v>
@@ -1207,25 +1217,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>43</v>
+      <c r="H8" s="11" t="s">
+        <v>182</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>20</v>
@@ -1234,7 +1244,7 @@
         <v>21</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>23</v>
@@ -1248,25 +1258,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>47</v>
+      <c r="H9" s="11" t="s">
+        <v>181</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>20</v>
@@ -1289,13 +1299,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>16</v>
@@ -1306,8 +1316,8 @@
       <c r="G10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>51</v>
+      <c r="H10" s="11" t="s">
+        <v>180</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>20</v>
@@ -1330,25 +1340,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>56</v>
+      <c r="H11" s="11" t="s">
+        <v>179</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -1371,25 +1381,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>60</v>
+      <c r="H12" s="11" t="s">
+        <v>178</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -1412,13 +1422,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>16</v>
@@ -1429,8 +1439,8 @@
       <c r="G13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>62</v>
+      <c r="H13" s="11" t="s">
+        <v>177</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>20</v>
@@ -1453,10 +1463,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>15</v>
@@ -1470,8 +1480,8 @@
       <c r="G14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>65</v>
+      <c r="H14" s="11" t="s">
+        <v>176</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>20</v>
@@ -1494,25 +1504,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>66</v>
+      <c r="H15" s="11" t="s">
+        <v>175</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>20</v>
@@ -1535,25 +1545,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>69</v>
+      <c r="H16" s="11" t="s">
+        <v>174</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>20</v>
@@ -1576,13 +1586,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>16</v>
@@ -1594,7 +1604,7 @@
         <v>18</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>20</v>
@@ -1603,7 +1613,7 @@
         <v>21</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L17" s="1" t="s">
         <v>23</v>
@@ -1617,25 +1627,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>74</v>
+      <c r="H18" s="11" t="s">
+        <v>173</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>20</v>
@@ -1658,25 +1668,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>75</v>
+      <c r="H19" s="11" t="s">
+        <v>172</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>20</v>
@@ -1699,13 +1709,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>16</v>
@@ -1717,7 +1727,7 @@
         <v>18</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>20</v>
@@ -1726,7 +1736,7 @@
         <v>21</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L20" s="1" t="s">
         <v>23</v>
@@ -1740,10 +1750,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>15</v>
@@ -1757,8 +1767,8 @@
       <c r="G21" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>80</v>
+      <c r="H21" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>20</v>
@@ -1767,7 +1777,7 @@
         <v>21</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L21" s="1" t="s">
         <v>23</v>
@@ -1781,25 +1791,25 @@
         <v>21</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" s="8">
-        <v>52000</v>
+        <v>68</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>85</v>
+        <v>70</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>171</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>20</v>
@@ -1808,10 +1818,10 @@
         <v>21</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="M22" s="10">
         <v>46099</v>
@@ -1822,25 +1832,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23" s="8">
-        <v>39000</v>
+        <v>74</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>52</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>91</v>
+      <c r="H23" s="11" t="s">
+        <v>169</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>20</v>
@@ -1863,13 +1873,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D24" s="8">
-        <v>13000</v>
+        <v>64</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>144</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>16</v>
@@ -1881,7 +1891,7 @@
         <v>18</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>20</v>
@@ -1890,7 +1900,7 @@
         <v>21</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L24" s="8" t="s">
         <v>23</v>
@@ -1904,10 +1914,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D25" s="8">
         <v>13000</v>
@@ -1921,8 +1931,8 @@
       <c r="G25" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>95</v>
+      <c r="H25" s="11" t="s">
+        <v>168</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>20</v>
@@ -1945,10 +1955,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D26" s="8">
         <v>13000</v>
@@ -1962,8 +1972,8 @@
       <c r="G26" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H26" s="8" t="s">
-        <v>96</v>
+      <c r="H26" s="11" t="s">
+        <v>166</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>20</v>
@@ -1972,7 +1982,7 @@
         <v>21</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L26" s="8" t="s">
         <v>23</v>
@@ -1986,10 +1996,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D27" s="8">
         <v>19000</v>
@@ -2003,8 +2013,8 @@
       <c r="G27" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H27" s="8" t="s">
-        <v>98</v>
+      <c r="H27" s="11" t="s">
+        <v>167</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>20</v>
@@ -2013,7 +2023,7 @@
         <v>21</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L27" s="8" t="s">
         <v>23</v>
@@ -2027,10 +2037,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D28" s="8">
         <v>18000</v>
@@ -2039,13 +2049,13 @@
         <v>16</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H28" s="8" t="s">
-        <v>102</v>
+      <c r="H28" s="11" t="s">
+        <v>165</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>20</v>
@@ -2054,7 +2064,7 @@
         <v>21</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L28" s="8" t="s">
         <v>23</v>
@@ -2068,10 +2078,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D29" s="8">
         <v>19000</v>
@@ -2085,8 +2095,8 @@
       <c r="G29" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H29" s="8" t="s">
-        <v>104</v>
+      <c r="H29" s="11" t="s">
+        <v>164</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>20</v>
@@ -2109,10 +2119,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D30" s="8">
         <v>19000</v>
@@ -2126,8 +2136,8 @@
       <c r="G30" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H30" s="8" t="s">
-        <v>106</v>
+      <c r="H30" s="11" t="s">
+        <v>163</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>20</v>
@@ -2136,7 +2146,7 @@
         <v>21</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L30" s="8" t="s">
         <v>23</v>
@@ -2150,10 +2160,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D31" s="8">
         <v>32000</v>
@@ -2162,13 +2172,13 @@
         <v>16</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="8" t="s">
-        <v>109</v>
+      <c r="H31" s="11" t="s">
+        <v>162</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>20</v>
@@ -2191,10 +2201,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D32" s="8">
         <v>28000</v>
@@ -2203,13 +2213,13 @@
         <v>16</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H32" s="8" t="s">
-        <v>111</v>
+      <c r="H32" s="11" t="s">
+        <v>161</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>20</v>
@@ -2218,7 +2228,7 @@
         <v>21</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L32" s="8" t="s">
         <v>23</v>
@@ -2232,10 +2242,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D33" s="8">
         <v>21000</v>
@@ -2244,13 +2254,13 @@
         <v>16</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>115</v>
+        <v>90</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>160</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>20</v>
@@ -2259,10 +2269,10 @@
         <v>21</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L33" s="8" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="M33" s="10">
         <v>46099</v>
@@ -2273,10 +2283,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D34" s="8">
         <v>24000</v>
@@ -2285,13 +2295,13 @@
         <v>16</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>20</v>
@@ -2300,10 +2310,10 @@
         <v>21</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L34" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M34" s="10">
         <v>46099</v>
@@ -2314,10 +2324,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D35" s="8">
         <v>24000</v>
@@ -2326,13 +2336,13 @@
         <v>16</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>20</v>
@@ -2344,7 +2354,7 @@
         <v>22</v>
       </c>
       <c r="L35" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M35" s="10">
         <v>46099</v>
@@ -2355,10 +2365,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D36" s="8">
         <v>24000</v>
@@ -2367,13 +2377,13 @@
         <v>16</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>20</v>
@@ -2382,10 +2392,10 @@
         <v>21</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="L36" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M36" s="10">
         <v>46099</v>
@@ -2396,10 +2406,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D37" s="8">
         <v>24000</v>
@@ -2408,13 +2418,13 @@
         <v>16</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>20</v>
@@ -2423,10 +2433,10 @@
         <v>21</v>
       </c>
       <c r="K37" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L37" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M37" s="10">
         <v>46099</v>
@@ -2437,10 +2447,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D38" s="8">
         <v>24000</v>
@@ -2449,13 +2459,13 @@
         <v>16</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>20</v>
@@ -2464,10 +2474,10 @@
         <v>21</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L38" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M38" s="10">
         <v>46099</v>
@@ -2478,10 +2488,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D39" s="8">
         <v>24000</v>
@@ -2490,13 +2500,13 @@
         <v>16</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>20</v>
@@ -2505,10 +2515,10 @@
         <v>21</v>
       </c>
       <c r="K39" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L39" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M39" s="10">
         <v>46099</v>
@@ -2519,10 +2529,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D40" s="8">
         <v>24000</v>
@@ -2531,13 +2541,13 @@
         <v>16</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>20</v>
@@ -2546,10 +2556,10 @@
         <v>21</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L40" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M40" s="10">
         <v>46099</v>
@@ -2560,10 +2570,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D41" s="8">
         <v>24000</v>
@@ -2572,13 +2582,13 @@
         <v>16</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>20</v>
@@ -2590,7 +2600,7 @@
         <v>26</v>
       </c>
       <c r="L41" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M41" s="10">
         <v>46099</v>
@@ -2601,10 +2611,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D42" s="8">
         <v>24000</v>
@@ -2613,13 +2623,13 @@
         <v>16</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>20</v>
@@ -2628,10 +2638,10 @@
         <v>21</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L42" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M42" s="10">
         <v>46099</v>
@@ -2642,10 +2652,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D43" s="8">
         <v>24000</v>
@@ -2654,13 +2664,13 @@
         <v>16</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H43" s="11" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>20</v>
@@ -2669,10 +2679,10 @@
         <v>21</v>
       </c>
       <c r="K43" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L43" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M43" s="10">
         <v>46099</v>
@@ -2683,10 +2693,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D44" s="8">
         <v>24000</v>
@@ -2695,13 +2705,13 @@
         <v>16</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H44" s="11" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>20</v>
@@ -2710,10 +2720,10 @@
         <v>21</v>
       </c>
       <c r="K44" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L44" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M44" s="10">
         <v>46099</v>
@@ -2724,10 +2734,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D45" s="8">
         <v>27000</v>
@@ -2736,13 +2746,13 @@
         <v>16</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H45" s="11" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>20</v>
@@ -2754,7 +2764,7 @@
         <v>22</v>
       </c>
       <c r="L45" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M45" s="10">
         <v>46099</v>
@@ -2765,10 +2775,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D46" s="8">
         <v>27000</v>
@@ -2777,13 +2787,13 @@
         <v>16</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H46" s="11" t="s">
-        <v>134</v>
+        <v>109</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>20</v>
@@ -2792,10 +2802,10 @@
         <v>21</v>
       </c>
       <c r="K46" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L46" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M46" s="10">
         <v>46099</v>
@@ -2806,10 +2816,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D47" s="8">
         <v>20000</v>
@@ -2818,13 +2828,13 @@
         <v>16</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>20</v>
@@ -2836,7 +2846,7 @@
         <v>26</v>
       </c>
       <c r="L47" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M47" s="10">
         <v>46099</v>
@@ -2847,10 +2857,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D48" s="8">
         <v>20000</v>
@@ -2859,13 +2869,13 @@
         <v>16</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>20</v>
@@ -2874,10 +2884,10 @@
         <v>21</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L48" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M48" s="10">
         <v>46099</v>
@@ -2888,10 +2898,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D49" s="8">
         <v>20000</v>
@@ -2900,13 +2910,13 @@
         <v>16</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H49" s="11" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>20</v>
@@ -2915,10 +2925,10 @@
         <v>21</v>
       </c>
       <c r="K49" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L49" s="8" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M49" s="10">
         <v>46099</v>
@@ -2929,10 +2939,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D50" s="8">
         <v>55000</v>
@@ -2941,13 +2951,13 @@
         <v>16</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H50" s="11" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>20</v>
@@ -2956,10 +2966,10 @@
         <v>21</v>
       </c>
       <c r="K50" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L50" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M50" s="10">
         <v>46099</v>
@@ -2970,10 +2980,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D51" s="8">
         <v>55000</v>
@@ -2982,13 +2992,13 @@
         <v>16</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G51" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H51" s="11" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>20</v>
@@ -2997,10 +3007,10 @@
         <v>21</v>
       </c>
       <c r="K51" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L51" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M51" s="10">
         <v>46099</v>
@@ -3011,10 +3021,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D52" s="8">
         <v>55000</v>
@@ -3023,13 +3033,13 @@
         <v>16</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G52" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H52" s="11" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>20</v>
@@ -3038,10 +3048,10 @@
         <v>21</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L52" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M52" s="10">
         <v>46099</v>
@@ -3052,10 +3062,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D53" s="8">
         <v>65000</v>
@@ -3064,13 +3074,13 @@
         <v>16</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H53" s="11" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>20</v>
@@ -3082,7 +3092,7 @@
         <v>22</v>
       </c>
       <c r="L53" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M53" s="10">
         <v>46099</v>
@@ -3093,10 +3103,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D54" s="8">
         <v>60000</v>
@@ -3105,13 +3115,13 @@
         <v>16</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H54" s="11" t="s">
-        <v>148</v>
+        <v>123</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>20</v>
@@ -3120,10 +3130,10 @@
         <v>21</v>
       </c>
       <c r="K54" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L54" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M54" s="10">
         <v>46099</v>
@@ -3134,10 +3144,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D55" s="8">
         <v>60000</v>
@@ -3146,13 +3156,13 @@
         <v>16</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>20</v>
@@ -3161,10 +3171,10 @@
         <v>21</v>
       </c>
       <c r="K55" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L55" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M55" s="10">
         <v>46099</v>
@@ -3175,10 +3185,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="D56" s="8">
         <v>60000</v>
@@ -3187,13 +3197,13 @@
         <v>16</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>20</v>
@@ -3202,10 +3212,10 @@
         <v>21</v>
       </c>
       <c r="K56" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L56" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M56" s="10">
         <v>46099</v>
@@ -3216,10 +3226,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D57" s="8">
         <v>55000</v>
@@ -3228,13 +3238,13 @@
         <v>16</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H57" s="8" t="s">
-        <v>153</v>
+      <c r="H57" s="11" t="s">
+        <v>149</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>20</v>
@@ -3243,10 +3253,10 @@
         <v>21</v>
       </c>
       <c r="K57" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L57" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M57" s="10">
         <v>46099</v>
@@ -3257,10 +3267,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D58" s="8">
         <v>64000</v>
@@ -3269,13 +3279,13 @@
         <v>16</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="G58" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H58" s="8" t="s">
-        <v>155</v>
+        <v>70</v>
+      </c>
+      <c r="H58" s="11" t="s">
+        <v>150</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>20</v>
@@ -3287,7 +3297,7 @@
         <v>22</v>
       </c>
       <c r="L58" s="8" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="M58" s="10">
         <v>46099</v>
@@ -3298,10 +3308,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D59" s="8">
         <v>64000</v>
@@ -3310,13 +3320,13 @@
         <v>16</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H59" s="8" t="s">
-        <v>157</v>
+        <v>70</v>
+      </c>
+      <c r="H59" s="11" t="s">
+        <v>151</v>
       </c>
       <c r="I59" s="8" t="s">
         <v>20</v>
@@ -3325,10 +3335,10 @@
         <v>21</v>
       </c>
       <c r="K59" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L59" s="8" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="M59" s="10">
         <v>46099</v>
@@ -3339,10 +3349,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D60" s="8">
         <v>64000</v>
@@ -3351,13 +3361,13 @@
         <v>16</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G60" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H60" s="8" t="s">
-        <v>158</v>
+        <v>70</v>
+      </c>
+      <c r="H60" s="11" t="s">
+        <v>152</v>
       </c>
       <c r="I60" s="8" t="s">
         <v>20</v>
@@ -3366,10 +3376,10 @@
         <v>21</v>
       </c>
       <c r="K60" s="8" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="L60" s="8" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="M60" s="10">
         <v>46099</v>
@@ -3380,10 +3390,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D61" s="8">
         <v>64000</v>
@@ -3392,13 +3402,13 @@
         <v>16</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H61" s="8" t="s">
-        <v>160</v>
+        <v>70</v>
+      </c>
+      <c r="H61" s="11" t="s">
+        <v>153</v>
       </c>
       <c r="I61" s="8" t="s">
         <v>20</v>
@@ -3407,10 +3417,10 @@
         <v>21</v>
       </c>
       <c r="K61" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L61" s="8" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
       <c r="M61" s="10">
         <v>46099</v>
@@ -3421,10 +3431,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D62" s="8">
         <v>36000</v>
@@ -3433,13 +3443,13 @@
         <v>16</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H62" s="8" t="s">
-        <v>161</v>
+        <v>70</v>
+      </c>
+      <c r="H62" s="11" t="s">
+        <v>154</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>20</v>
@@ -3448,10 +3458,10 @@
         <v>21</v>
       </c>
       <c r="K62" s="8" t="s">
-        <v>162</v>
+        <v>131</v>
       </c>
       <c r="L62" s="8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="M62" s="10">
         <v>46099</v>
@@ -3462,10 +3472,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D63" s="8">
         <v>36000</v>
@@ -3474,13 +3484,13 @@
         <v>16</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H63" s="8" t="s">
-        <v>164</v>
+        <v>70</v>
+      </c>
+      <c r="H63" s="11" t="s">
+        <v>155</v>
       </c>
       <c r="I63" s="8" t="s">
         <v>20</v>
@@ -3489,10 +3499,10 @@
         <v>21</v>
       </c>
       <c r="K63" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L63" s="8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="M63" s="10">
         <v>46099</v>
@@ -3503,10 +3513,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D64" s="8">
         <v>36000</v>
@@ -3515,13 +3525,13 @@
         <v>16</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H64" s="8" t="s">
-        <v>165</v>
+        <v>70</v>
+      </c>
+      <c r="H64" s="11" t="s">
+        <v>156</v>
       </c>
       <c r="I64" s="8" t="s">
         <v>20</v>
@@ -3530,10 +3540,10 @@
         <v>21</v>
       </c>
       <c r="K64" s="8" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="L64" s="8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="M64" s="10">
         <v>46099</v>
@@ -3544,10 +3554,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D65" s="8">
         <v>36000</v>
@@ -3556,13 +3566,13 @@
         <v>16</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H65" s="8" t="s">
-        <v>166</v>
+        <v>70</v>
+      </c>
+      <c r="H65" s="11" t="s">
+        <v>158</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>20</v>
@@ -3571,10 +3581,10 @@
         <v>21</v>
       </c>
       <c r="K65" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L65" s="8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="M65" s="10">
         <v>46099</v>
@@ -3585,10 +3595,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D66" s="8">
         <v>36000</v>
@@ -3597,13 +3607,13 @@
         <v>16</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G66" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H66" s="8" t="s">
-        <v>167</v>
+        <v>70</v>
+      </c>
+      <c r="H66" s="11" t="s">
+        <v>157</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>20</v>
@@ -3612,10 +3622,10 @@
         <v>21</v>
       </c>
       <c r="K66" s="8" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
       <c r="L66" s="8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="M66" s="10">
         <v>46099</v>
@@ -3626,10 +3636,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D67" s="8">
         <v>21000</v>
@@ -3638,13 +3648,13 @@
         <v>16</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H67" s="11" t="s">
-        <v>168</v>
+        <v>133</v>
       </c>
       <c r="I67" s="8" t="s">
         <v>20</v>
@@ -3656,7 +3666,7 @@
         <v>26</v>
       </c>
       <c r="L67" s="8" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="M67" s="10">
         <v>46099</v>
@@ -3667,10 +3677,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="D68" s="8">
         <v>21000</v>
@@ -3679,13 +3689,13 @@
         <v>16</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H68" s="11" t="s">
-        <v>169</v>
+        <v>134</v>
       </c>
       <c r="I68" s="8" t="s">
         <v>20</v>
@@ -3697,7 +3707,7 @@
         <v>26</v>
       </c>
       <c r="L68" s="8" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="M68" s="10">
         <v>46099</v>
@@ -3708,10 +3718,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D69" s="8">
         <v>32000</v>
@@ -3720,13 +3730,13 @@
         <v>16</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H69" s="8" t="s">
-        <v>170</v>
+        <v>70</v>
+      </c>
+      <c r="H69" s="11" t="s">
+        <v>159</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>20</v>
@@ -3735,10 +3745,10 @@
         <v>21</v>
       </c>
       <c r="K69" s="8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L69" s="8" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="M69" s="10">
         <v>46099</v>
@@ -3749,10 +3759,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D70" s="8">
         <v>63000</v>
@@ -3761,13 +3771,13 @@
         <v>16</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="G70" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H70" s="8" t="s">
-        <v>174</v>
+        <v>138</v>
       </c>
       <c r="I70" s="8" t="s">
         <v>20</v>
@@ -3776,10 +3786,10 @@
         <v>21</v>
       </c>
       <c r="K70" s="8" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L70" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M70" s="10">
         <v>46099</v>
@@ -3790,10 +3800,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D71" s="8">
         <v>36000</v>
@@ -3802,13 +3812,13 @@
         <v>16</v>
       </c>
       <c r="F71" s="9" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="G71" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H71" s="8" t="s">
-        <v>176</v>
+        <v>147</v>
       </c>
       <c r="I71" s="8" t="s">
         <v>20</v>
@@ -3820,7 +3830,7 @@
         <v>22</v>
       </c>
       <c r="L71" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M71" s="10">
         <v>46099</v>
@@ -3831,10 +3841,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D72" s="8">
         <v>36000</v>
@@ -3843,13 +3853,13 @@
         <v>16</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G72" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H72" s="8" t="s">
-        <v>177</v>
+      <c r="H72" s="11" t="s">
+        <v>148</v>
       </c>
       <c r="I72" s="8" t="s">
         <v>20</v>
@@ -3861,7 +3871,7 @@
         <v>22</v>
       </c>
       <c r="L72" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M72" s="10">
         <v>46099</v>
@@ -3872,10 +3882,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>179</v>
+        <v>141</v>
       </c>
       <c r="D73" s="8">
         <v>25000</v>
@@ -3884,13 +3894,13 @@
         <v>16</v>
       </c>
       <c r="F73" s="9" t="s">
-        <v>180</v>
+        <v>142</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H73" s="8" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="I73" s="8" t="s">
         <v>20</v>
@@ -3902,7 +3912,7 @@
         <v>22</v>
       </c>
       <c r="L73" s="8" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="M73" s="10">
         <v>46099</v>
@@ -4950,6 +4960,43 @@
     <hyperlink ref="H56" r:id="rId30" xr:uid="{1D3BB45C-C7E9-174F-8F72-A00DC3563F84}"/>
     <hyperlink ref="H67" r:id="rId31" xr:uid="{BCA705D2-FDC0-1C4D-8B19-E359DFC50FFF}"/>
     <hyperlink ref="H68" r:id="rId32" xr:uid="{8E93EE4F-9052-A844-916D-D6F1C62AAF47}"/>
+    <hyperlink ref="H72" r:id="rId33" display="https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835622/tg-products/xpswgt46xryxgyiizb5q.jpg" xr:uid="{475D28CB-5EA7-E445-8A81-29A0842BBCF9}"/>
+    <hyperlink ref="H57" r:id="rId34" xr:uid="{11BE95AC-3563-5443-95E9-B98D2CA4FBE3}"/>
+    <hyperlink ref="H58" r:id="rId35" xr:uid="{A8489FD4-C980-F74A-8425-1EE6A56010C1}"/>
+    <hyperlink ref="H59" r:id="rId36" xr:uid="{FE9A185F-5B84-CE46-8AE1-69C1CDF24D3D}"/>
+    <hyperlink ref="H60" r:id="rId37" xr:uid="{E91E591B-05DD-FF42-8BDC-97E775FD0049}"/>
+    <hyperlink ref="H61" r:id="rId38" xr:uid="{C4B3F011-F0E2-6948-986C-9E061116FB9E}"/>
+    <hyperlink ref="H62" r:id="rId39" xr:uid="{AE825DE9-98AE-C643-9AC2-973B335AA197}"/>
+    <hyperlink ref="H63" r:id="rId40" xr:uid="{FB2EDF1A-C2DB-1A42-9895-A5C7022D920F}"/>
+    <hyperlink ref="H64" r:id="rId41" xr:uid="{35B5D7D5-DEF9-C448-9C05-4B69FA7BCE70}"/>
+    <hyperlink ref="H66" r:id="rId42" xr:uid="{D46A5009-693F-2D41-848D-3F9BC95858DD}"/>
+    <hyperlink ref="H65" r:id="rId43" xr:uid="{FD4AF6E4-DC4F-364C-9F4B-7A9B4F54ECA9}"/>
+    <hyperlink ref="H69" r:id="rId44" xr:uid="{AE457894-C6E1-5243-A590-74C71268C011}"/>
+    <hyperlink ref="H33" r:id="rId45" xr:uid="{594321F7-9F4D-1047-B12A-2CB991EA0316}"/>
+    <hyperlink ref="H32" r:id="rId46" xr:uid="{0E5E614B-ADFA-9248-AD14-BF44811E2B60}"/>
+    <hyperlink ref="H31" r:id="rId47" xr:uid="{E4F06C48-6C84-9A47-AD46-0A10654BEB25}"/>
+    <hyperlink ref="H30" r:id="rId48" xr:uid="{7BF14278-EE98-E945-B1BB-B07165BCBF97}"/>
+    <hyperlink ref="H29" r:id="rId49" xr:uid="{83F817CC-B7C6-F245-B4F8-C8CEAB7084E2}"/>
+    <hyperlink ref="H28" r:id="rId50" xr:uid="{502C56AC-B5B1-144D-AB5C-E2528F8C8A5C}"/>
+    <hyperlink ref="H26" r:id="rId51" xr:uid="{448202B5-2D9F-214E-B534-6C652898B069}"/>
+    <hyperlink ref="H27" r:id="rId52" xr:uid="{BACD3E75-FC57-8D4C-AE21-7CCBE55393F5}"/>
+    <hyperlink ref="H25" r:id="rId53" xr:uid="{41CAA107-54AE-7245-9C76-7AFD8B093580}"/>
+    <hyperlink ref="H23" r:id="rId54" xr:uid="{F83164A8-CB7B-714C-9673-C5DB38B8726A}"/>
+    <hyperlink ref="H21" r:id="rId55" xr:uid="{3720409C-694C-F24F-BC82-3BF533187DB5}"/>
+    <hyperlink ref="H22" r:id="rId56" xr:uid="{3BBA25AD-84A8-F545-B7C6-A8BCD20C0193}"/>
+    <hyperlink ref="H19" r:id="rId57" xr:uid="{1C22F573-F7B1-984F-9769-5F0002B9CE9B}"/>
+    <hyperlink ref="H18" r:id="rId58" xr:uid="{BCBFE71D-030F-AE4E-9178-AEED804BA399}"/>
+    <hyperlink ref="H16" r:id="rId59" xr:uid="{C7540697-781F-AA46-AB0D-81D2BEE98CD5}"/>
+    <hyperlink ref="H15" r:id="rId60" xr:uid="{5208BA8B-3351-F340-9C08-AE2F16F7BF62}"/>
+    <hyperlink ref="H14" r:id="rId61" xr:uid="{54921A81-B696-EC40-B773-DA445DA1556F}"/>
+    <hyperlink ref="H13" r:id="rId62" xr:uid="{1F04152C-9072-B242-A5CF-D6AFA14CABA5}"/>
+    <hyperlink ref="H12" r:id="rId63" xr:uid="{8B155CE8-066E-3241-82E3-B6202D63041B}"/>
+    <hyperlink ref="H11" r:id="rId64" xr:uid="{5E8AC82B-CABC-A444-BE5F-1AD24F1D1839}"/>
+    <hyperlink ref="H10" r:id="rId65" xr:uid="{4C0B6705-6286-A741-BB53-1B9062FF53C0}"/>
+    <hyperlink ref="H9" r:id="rId66" xr:uid="{C1C9F9B3-829D-E545-AF66-013A250A217E}"/>
+    <hyperlink ref="H8" r:id="rId67" xr:uid="{BC392C16-44E5-0247-9603-E28D1664E0BC}"/>
+    <hyperlink ref="H7" r:id="rId68" xr:uid="{BEC9B471-A176-CF47-9FCA-E2FA242AA85A}"/>
+    <hyperlink ref="H5" r:id="rId69" xr:uid="{97C5CAB9-0FD9-2E44-87D6-AEDA82ABBA70}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update products and order recipient
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a/ЛСсайт/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2D99DD-513E-7C48-BBEA-C430C895E7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0D2ACE-2770-6F43-9720-9CD3B078663E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="255">
   <si>
     <t>id</t>
   </si>
@@ -466,9 +466,6 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835561/tg-products/djmln37ynprbvnw9j3kf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835567/tg-products/bcloy4laepu7xjnximux.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835622/tg-products/xpswgt46xryxgyiizb5q.jpg,  https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835577/tg-products/ms4qzopjvfmnvxe4fyql.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835610/tg-products/ry6zindmjsnornscgrre.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835614/tg-products/maa475djsqbflpsu43uq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835617/tg-products/xfa7pbpame6l5jhjcy2r.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773833036/tg-products/fwfq56v1fhvye5vn7tca.jpg</t>
   </si>
   <si>
@@ -575,6 +572,219 @@
   </si>
   <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773657069/tg-products/bhgxysknyx1l2jk9u3rn.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835622/tg-products/xpswgt46xryxgyiizb5q.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835610/tg-products/ry6zindmjsnornscgrre.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835614/tg-products/maa475djsqbflpsu43uq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773835617/tg-products/xfa7pbpame6l5jhjcy2r.jpg</t>
+  </si>
+  <si>
+    <t>Футболка Loewe</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773914971/tg-products/d1salpeehkzhhihxoanc.jpg</t>
+  </si>
+  <si>
+    <t>Рубашка Dior</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773914978/tg-products/vb1w8lhiclcmlq3sdyr1.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773914986/tg-products/z4wejuwnxlxhnczb0o21.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773914995/tg-products/plvk8isxl2lp6o6uquml.jpg</t>
+  </si>
+  <si>
+    <t>Футболка Hermes</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915004/tg-products/bjyujibnpchdpqt3l4bg.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915010/tg-products/akcys7bv9vxcmdeppsuk.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915133/tg-products/qq6oo9af9mwumggnc1qz.jpg</t>
+  </si>
+  <si>
+    <t>Сумка Chanel</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915641/tg-products/stkyhzzdkuh1cgimaizl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915643/tg-products/tzko9pcwffbbwbbufkfv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915648/tg-products/uf0pp82dkddefxuqld1s.jpg</t>
+  </si>
+  <si>
+    <t>23х14х6 см</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915701/tg-products/bvup6c9kmi4zlzidrgyq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915713/tg-products/qmmjhrb4i7hnshqgbiyb.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915721/tg-products/rqlei70guawavf6fhzjo.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915768/tg-products/xalpgyleamdxmb1oyzq9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915771/tg-products/fumo4n1kyawnlcva1nif.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915786/tg-products/c53oo1tsfepwatxfoqdc.jpg</t>
+  </si>
+  <si>
+    <t>17х14х8 см</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915974/tg-products/okpiwinqf4jcsf7nr3hf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915983/tg-products/hqs27dixwbs9zfsletjk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915992/tg-products/klvb2yk28squrw4eqcoe.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916026/tg-products/v3bzscftxxtfkok5cdaf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916040/tg-products/cul4h6zea2sonxd1lgxf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916055/tg-products/mffin77lcud3f2op2cyd.jpg</t>
+  </si>
+  <si>
+    <t>22х20х13 см</t>
+  </si>
+  <si>
+    <t>Материал ткань</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916102/tg-products/fnje0ov6zeyrfokmxdks.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916113/tg-products/cgpw0axs1slqut7jrnrk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916132/tg-products/tbbqejtlrdnzpynr0nws.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916086/tg-products/sddmxitn3mxmgthy2cp1.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916093/tg-products/wxfglpoym9jkav8kz9kf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916138/tg-products/qlzplygyrsjonuc6kiqk.jpg</t>
+  </si>
+  <si>
+    <t>Рюкзак Miumiu</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916432/tg-products/l1wohpgzi9o8rnu80flv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916436/tg-products/mrmuffh9c6uvbhg9s7rk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916445/tg-products/ilk8cs62va6xydzdmstw.jpg</t>
+  </si>
+  <si>
+    <t>30х25х13 см</t>
+  </si>
+  <si>
+    <t>Материал черный</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916474/tg-products/afceszq8os8lberkmalm.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916485/tg-products/p9uxynpkqbn2efirha2t.jpg</t>
+  </si>
+  <si>
+    <t>Сумка Miumiu</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916495/tg-products/rdgkfra33efqfoebrgka.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916513/tg-products/e0ebomobixo7w1mjg5jk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916521/tg-products/l9jpafud4kicigrgexwc.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916526/tg-products/lfhgnrx8fx2bayw4d0ve.jpg</t>
+  </si>
+  <si>
+    <t>44х23х14 см</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916555/tg-products/pwqnaichbddjbn9oapdd.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916564/tg-products/znxg24dqz9iogwltnsg8.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916590/tg-products/ot81lsalffufeiq8rks1.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916922/tg-products/eootmyjtcnsi4yr4m62z.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916929/tg-products/fotezp5mzile8hxif7dl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916940/tg-products/ghkrsbfqxkpdjudellin.jpg</t>
+  </si>
+  <si>
+    <t>33х19х5 см</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916978/tg-products/l1haqfjdigfv4gznyeea.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg</t>
+  </si>
+  <si>
+    <t>серый</t>
+  </si>
+  <si>
+    <t>Топ Fendi</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933748/tg-products/xdb2jkfqk6wesecqdolt.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933749/tg-products/mgcrk3utqbezfs4ixztw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933756/tg-products/yiu9q66cs6mwcfahauri.jpg</t>
+  </si>
+  <si>
+    <t>Рубашка Fendi</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933794/tg-products/bdl0j9ioh5mayldrjmfw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933795/tg-products/enspkgek73kduyxzd0e9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933796/tg-products/hvt9ykb7wv9vwn2fegto.jpg</t>
+  </si>
+  <si>
+    <t>Свитер Hermes</t>
+  </si>
+  <si>
+    <t>Материал хлопок и шелк</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933843/tg-products/tqqmzddc6gtpkhmpksex.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933844/tg-products/zezm4sstdkbsfkloqbx4.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933846/tg-products/oc7cxfwca0ogmwaem0wp.jpg</t>
+  </si>
+  <si>
+    <t>Поло Prada</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933876/tg-products/fuldr5oxwjl4ofjtyvb5.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933881/tg-products/zxsbuqp1zi6fmudrcrge.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933882/tg-products/ibvz2vhk5zjttfjncoju.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933931/tg-products/y3preqgf4yrmzvjiabuh.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933932/tg-products/ko7czxgykv0usognjmff.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933933/tg-products/bnlf6iyyg9u6mlqciplj.jpg</t>
+  </si>
+  <si>
+    <t>Платье Louis Vuitton</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773934457/tg-products/ltj8m2vwgmhol94h9ood.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940115/tg-products/zynb4me8jy8291jyhwo9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940116/tg-products/guma9ms2hjqdeypzy08k.jpg</t>
+  </si>
+  <si>
+    <t>Лоферы Loro Piana</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940128/tg-products/rjupb6z4rvxu26o3iptv.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940133/tg-products/buiap7kz84pnau6b7d1e.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940139/tg-products/xuxunnpxdjvvdhyyvadl.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940149/tg-products/kxqmw1dnvgaygedtqeaw.jpg</t>
+  </si>
+  <si>
+    <t>Лоферы Chanel</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940167/tg-products/vfqr3udjudlkjyohduwn.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940188/tg-products/epxsyy8fjnuhfzn9rirj.jpg</t>
+  </si>
+  <si>
+    <t>Ботинки Celine</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940219/tg-products/l3e2d1kkyzdxysui3ov2.jpg</t>
+  </si>
+  <si>
+    <t>Ботинки Chanel</t>
+  </si>
+  <si>
+    <t>Материал резина</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940244/tg-products/l8nrk9ffjse9je0bh93x.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940263/tg-products/htcis0dfvogocejsezlt.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940338/tg-products/xahkvzjmg8ygpigezbav.jpg</t>
+  </si>
+  <si>
+    <t>22х15х7 см</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940418/tg-products/o9edgik4to8axapcxs0d.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940424/tg-products/pogpzdov1xuj4diavlax.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940439/tg-products/wzb88maxjbg22dqj3q4g.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940473/tg-products/towwzks0ieiqlxisqeue.jpg</t>
+  </si>
+  <si>
+    <t>17х11х5 см</t>
+  </si>
+  <si>
+    <t>Fendi</t>
+  </si>
+  <si>
+    <t>Louis Vuitton</t>
   </si>
 </sst>
 </file>
@@ -715,10 +925,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1112,7 +1318,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>20</v>
@@ -1194,7 +1400,7 @@
         <v>18</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
@@ -1235,7 +1441,7 @@
         <v>18</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>20</v>
@@ -1276,7 +1482,7 @@
         <v>18</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>20</v>
@@ -1317,7 +1523,7 @@
         <v>18</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>20</v>
@@ -1358,7 +1564,7 @@
         <v>18</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -1399,7 +1605,7 @@
         <v>18</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -1440,7 +1646,7 @@
         <v>18</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>20</v>
@@ -1481,7 +1687,7 @@
         <v>18</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>20</v>
@@ -1522,7 +1728,7 @@
         <v>18</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>20</v>
@@ -1563,7 +1769,7 @@
         <v>18</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>20</v>
@@ -1645,7 +1851,7 @@
         <v>18</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>20</v>
@@ -1686,7 +1892,7 @@
         <v>18</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>20</v>
@@ -1768,7 +1974,7 @@
         <v>18</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>20</v>
@@ -1809,7 +2015,7 @@
         <v>70</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>20</v>
@@ -1850,7 +2056,7 @@
         <v>18</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>20</v>
@@ -1932,7 +2138,7 @@
         <v>18</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>20</v>
@@ -1973,7 +2179,7 @@
         <v>18</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>20</v>
@@ -2014,7 +2220,7 @@
         <v>18</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>20</v>
@@ -2055,7 +2261,7 @@
         <v>18</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>20</v>
@@ -2096,7 +2302,7 @@
         <v>18</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>20</v>
@@ -2137,7 +2343,7 @@
         <v>18</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>20</v>
@@ -2178,7 +2384,7 @@
         <v>18</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>20</v>
@@ -2219,7 +2425,7 @@
         <v>18</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>20</v>
@@ -2260,7 +2466,7 @@
         <v>90</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>20</v>
@@ -3244,7 +3450,7 @@
         <v>18</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>20</v>
@@ -3285,7 +3491,7 @@
         <v>70</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>20</v>
@@ -3326,7 +3532,7 @@
         <v>70</v>
       </c>
       <c r="H59" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I59" s="8" t="s">
         <v>20</v>
@@ -3367,7 +3573,7 @@
         <v>70</v>
       </c>
       <c r="H60" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I60" s="8" t="s">
         <v>20</v>
@@ -3408,7 +3614,7 @@
         <v>70</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I61" s="8" t="s">
         <v>20</v>
@@ -3449,7 +3655,7 @@
         <v>70</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>20</v>
@@ -3490,7 +3696,7 @@
         <v>70</v>
       </c>
       <c r="H63" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I63" s="8" t="s">
         <v>20</v>
@@ -3531,7 +3737,7 @@
         <v>70</v>
       </c>
       <c r="H64" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I64" s="8" t="s">
         <v>20</v>
@@ -3572,7 +3778,7 @@
         <v>70</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>20</v>
@@ -3613,7 +3819,7 @@
         <v>70</v>
       </c>
       <c r="H66" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>20</v>
@@ -3736,7 +3942,7 @@
         <v>70</v>
       </c>
       <c r="H69" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>20</v>
@@ -3859,7 +4065,7 @@
         <v>18</v>
       </c>
       <c r="H72" s="11" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="I72" s="8" t="s">
         <v>20</v>
@@ -3919,566 +4125,1646 @@
       </c>
     </row>
     <row r="74" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
-      <c r="E74" s="8"/>
-      <c r="F74" s="8"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="8"/>
-      <c r="I74" s="8"/>
-      <c r="J74" s="8"/>
-      <c r="K74" s="8"/>
-      <c r="L74" s="8"/>
-      <c r="M74" s="8"/>
+      <c r="A74" s="1">
+        <v>73</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D74" s="8">
+        <v>12000</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G74" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H74" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="I74" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J74" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K74" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L74" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M74" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="75" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="8"/>
-      <c r="I75" s="8"/>
-      <c r="J75" s="8"/>
-      <c r="K75" s="8"/>
-      <c r="L75" s="8"/>
-      <c r="M75" s="8"/>
+      <c r="A75" s="1">
+        <v>74</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" s="8">
+        <v>14000</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G75" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H75" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="I75" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J75" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K75" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L75" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M75" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="76" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
-      <c r="G76" s="8"/>
-      <c r="H76" s="8"/>
-      <c r="I76" s="8"/>
-      <c r="J76" s="8"/>
-      <c r="K76" s="8"/>
-      <c r="L76" s="8"/>
-      <c r="M76" s="8"/>
+      <c r="A76" s="1">
+        <v>75</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D76" s="8">
+        <v>12000</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H76" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="I76" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J76" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K76" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="L76" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M76" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="77" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="8"/>
-      <c r="F77" s="8"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="8"/>
-      <c r="I77" s="8"/>
-      <c r="J77" s="8"/>
-      <c r="K77" s="8"/>
-      <c r="L77" s="8"/>
-      <c r="M77" s="8"/>
+      <c r="A77" s="1">
+        <v>76</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" s="8">
+        <v>12000</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="I77" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J77" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K77" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L77" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M77" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="78" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B78" s="8"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="8"/>
-      <c r="F78" s="8"/>
-      <c r="G78" s="8"/>
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="8"/>
-      <c r="K78" s="8"/>
-      <c r="L78" s="8"/>
-      <c r="M78" s="8"/>
+      <c r="A78" s="1">
+        <v>77</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D78" s="8">
+        <v>13000</v>
+      </c>
+      <c r="E78" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F78" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H78" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J78" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K78" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L78" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M78" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="79" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="8"/>
-      <c r="I79" s="8"/>
-      <c r="J79" s="8"/>
-      <c r="K79" s="8"/>
-      <c r="L79" s="8"/>
-      <c r="M79" s="8"/>
+      <c r="A79" s="1">
+        <v>78</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D79" s="8">
+        <v>11000</v>
+      </c>
+      <c r="E79" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H79" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="I79" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J79" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K79" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L79" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M79" s="10">
+        <v>46100</v>
+      </c>
     </row>
     <row r="80" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B80" s="8"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
-      <c r="E80" s="8"/>
-      <c r="F80" s="8"/>
-      <c r="G80" s="8"/>
-      <c r="H80" s="8"/>
-      <c r="I80" s="8"/>
-      <c r="J80" s="8"/>
-      <c r="K80" s="8"/>
-      <c r="L80" s="8"/>
-      <c r="M80" s="8"/>
-    </row>
-    <row r="81" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B81" s="8"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="8"/>
-      <c r="F81" s="8"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="8"/>
-      <c r="I81" s="8"/>
-      <c r="J81" s="8"/>
-      <c r="K81" s="8"/>
-      <c r="L81" s="8"/>
-      <c r="M81" s="8"/>
-    </row>
-    <row r="82" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B82" s="8"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
-      <c r="E82" s="8"/>
-      <c r="F82" s="8"/>
-      <c r="G82" s="8"/>
-      <c r="H82" s="8"/>
-      <c r="I82" s="8"/>
-      <c r="J82" s="8"/>
-      <c r="K82" s="8"/>
-      <c r="L82" s="8"/>
-      <c r="M82" s="8"/>
-    </row>
-    <row r="83" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B83" s="8"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="8"/>
-      <c r="F83" s="8"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="8"/>
-      <c r="I83" s="8"/>
-      <c r="J83" s="8"/>
-      <c r="K83" s="8"/>
-      <c r="L83" s="8"/>
-      <c r="M83" s="8"/>
-    </row>
-    <row r="84" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="8"/>
-      <c r="I84" s="8"/>
-      <c r="J84" s="8"/>
-      <c r="K84" s="8"/>
-      <c r="L84" s="8"/>
-      <c r="M84" s="8"/>
-    </row>
-    <row r="85" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B85" s="8"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="8"/>
-      <c r="F85" s="8"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="8"/>
-      <c r="I85" s="8"/>
-      <c r="J85" s="8"/>
-      <c r="K85" s="8"/>
-      <c r="L85" s="8"/>
-      <c r="M85" s="8"/>
-    </row>
-    <row r="86" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B86" s="8"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="8"/>
-      <c r="F86" s="8"/>
-      <c r="G86" s="8"/>
-      <c r="H86" s="8"/>
-      <c r="I86" s="8"/>
-      <c r="J86" s="8"/>
-      <c r="K86" s="8"/>
-      <c r="L86" s="8"/>
-      <c r="M86" s="8"/>
-    </row>
-    <row r="87" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B87" s="8"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="8"/>
-      <c r="F87" s="8"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="8"/>
-      <c r="I87" s="8"/>
-      <c r="J87" s="8"/>
-      <c r="K87" s="8"/>
-      <c r="L87" s="8"/>
-      <c r="M87" s="8"/>
-    </row>
-    <row r="88" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B88" s="8"/>
-      <c r="C88" s="8"/>
-      <c r="D88" s="8"/>
-      <c r="E88" s="8"/>
-      <c r="F88" s="8"/>
-      <c r="G88" s="8"/>
-      <c r="H88" s="8"/>
-      <c r="I88" s="8"/>
-      <c r="J88" s="8"/>
-      <c r="K88" s="8"/>
-      <c r="L88" s="8"/>
-      <c r="M88" s="8"/>
-    </row>
-    <row r="89" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
-      <c r="E89" s="8"/>
-      <c r="F89" s="8"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="8"/>
-      <c r="I89" s="8"/>
-      <c r="J89" s="8"/>
-      <c r="K89" s="8"/>
-      <c r="L89" s="8"/>
-      <c r="M89" s="8"/>
-    </row>
-    <row r="90" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B90" s="8"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="8"/>
-      <c r="F90" s="8"/>
-      <c r="G90" s="8"/>
-      <c r="H90" s="8"/>
-      <c r="I90" s="8"/>
-      <c r="J90" s="8"/>
-      <c r="K90" s="8"/>
-      <c r="L90" s="8"/>
-      <c r="M90" s="8"/>
-    </row>
-    <row r="91" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="8"/>
-      <c r="F91" s="8"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="8"/>
-      <c r="I91" s="8"/>
-      <c r="J91" s="8"/>
-      <c r="K91" s="8"/>
-      <c r="L91" s="8"/>
-      <c r="M91" s="8"/>
-    </row>
-    <row r="92" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B92" s="8"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="8"/>
-      <c r="E92" s="8"/>
-      <c r="F92" s="8"/>
-      <c r="G92" s="8"/>
-      <c r="H92" s="8"/>
-      <c r="I92" s="8"/>
-      <c r="J92" s="8"/>
-      <c r="K92" s="8"/>
-      <c r="L92" s="8"/>
-      <c r="M92" s="8"/>
-    </row>
-    <row r="93" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B93" s="8"/>
-      <c r="C93" s="8"/>
-      <c r="D93" s="8"/>
-      <c r="E93" s="8"/>
-      <c r="F93" s="8"/>
-      <c r="G93" s="8"/>
-      <c r="H93" s="8"/>
-      <c r="I93" s="8"/>
-      <c r="J93" s="8"/>
-      <c r="K93" s="8"/>
-      <c r="L93" s="8"/>
-      <c r="M93" s="8"/>
-    </row>
-    <row r="94" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
-      <c r="G94" s="8"/>
-      <c r="H94" s="8"/>
-      <c r="I94" s="8"/>
-      <c r="J94" s="8"/>
-      <c r="K94" s="8"/>
-      <c r="L94" s="8"/>
-      <c r="M94" s="8"/>
-    </row>
-    <row r="95" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
-      <c r="E95" s="8"/>
-      <c r="F95" s="8"/>
-      <c r="G95" s="8"/>
-      <c r="H95" s="8"/>
-      <c r="I95" s="8"/>
-      <c r="J95" s="8"/>
-      <c r="K95" s="8"/>
-      <c r="L95" s="8"/>
-      <c r="M95" s="8"/>
-    </row>
-    <row r="96" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B96" s="8"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="8"/>
-      <c r="E96" s="8"/>
-      <c r="F96" s="8"/>
-      <c r="G96" s="8"/>
-      <c r="H96" s="8"/>
-      <c r="I96" s="8"/>
-      <c r="J96" s="8"/>
-      <c r="K96" s="8"/>
-      <c r="L96" s="8"/>
-      <c r="M96" s="8"/>
-    </row>
-    <row r="97" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B97" s="8"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="8"/>
-      <c r="E97" s="8"/>
-      <c r="F97" s="8"/>
-      <c r="G97" s="8"/>
-      <c r="H97" s="8"/>
-      <c r="I97" s="8"/>
-      <c r="J97" s="8"/>
-      <c r="K97" s="8"/>
-      <c r="L97" s="8"/>
-      <c r="M97" s="8"/>
-    </row>
-    <row r="98" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B98" s="8"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="8"/>
-      <c r="E98" s="8"/>
-      <c r="F98" s="8"/>
-      <c r="G98" s="8"/>
-      <c r="H98" s="8"/>
-      <c r="I98" s="8"/>
-      <c r="J98" s="8"/>
-      <c r="K98" s="8"/>
-      <c r="L98" s="8"/>
-      <c r="M98" s="8"/>
-    </row>
-    <row r="99" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="8"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="8"/>
-      <c r="I99" s="8"/>
-      <c r="J99" s="8"/>
-      <c r="K99" s="8"/>
-      <c r="L99" s="8"/>
-      <c r="M99" s="8"/>
-    </row>
-    <row r="100" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="8"/>
-      <c r="G100" s="8"/>
-      <c r="H100" s="8"/>
-      <c r="I100" s="8"/>
-      <c r="J100" s="8"/>
-      <c r="K100" s="8"/>
-      <c r="L100" s="8"/>
-      <c r="M100" s="8"/>
-    </row>
-    <row r="101" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B101" s="8"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="8"/>
-      <c r="E101" s="8"/>
-      <c r="F101" s="8"/>
-      <c r="G101" s="8"/>
-      <c r="H101" s="8"/>
-      <c r="I101" s="8"/>
-      <c r="J101" s="8"/>
-      <c r="K101" s="8"/>
-      <c r="L101" s="8"/>
-      <c r="M101" s="8"/>
-    </row>
-    <row r="102" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B102" s="8"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="8"/>
-      <c r="E102" s="8"/>
-      <c r="F102" s="8"/>
-      <c r="G102" s="8"/>
-      <c r="H102" s="8"/>
-      <c r="I102" s="8"/>
-      <c r="J102" s="8"/>
-      <c r="K102" s="8"/>
-      <c r="L102" s="8"/>
-      <c r="M102" s="8"/>
-    </row>
-    <row r="103" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B103" s="8"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="8"/>
-      <c r="E103" s="8"/>
-      <c r="F103" s="8"/>
-      <c r="G103" s="8"/>
-      <c r="H103" s="8"/>
-      <c r="I103" s="8"/>
-      <c r="J103" s="8"/>
-      <c r="K103" s="8"/>
-      <c r="L103" s="8"/>
-      <c r="M103" s="8"/>
-    </row>
-    <row r="104" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B104" s="8"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
-      <c r="F104" s="8"/>
-      <c r="G104" s="8"/>
-      <c r="H104" s="8"/>
-      <c r="I104" s="8"/>
-      <c r="J104" s="8"/>
-      <c r="K104" s="8"/>
-      <c r="L104" s="8"/>
-      <c r="M104" s="8"/>
-    </row>
-    <row r="105" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B105" s="8"/>
-      <c r="C105" s="8"/>
-      <c r="D105" s="8"/>
-      <c r="E105" s="8"/>
-      <c r="F105" s="8"/>
-      <c r="G105" s="8"/>
-      <c r="H105" s="8"/>
-      <c r="I105" s="8"/>
-      <c r="J105" s="8"/>
-      <c r="K105" s="8"/>
-      <c r="L105" s="8"/>
-      <c r="M105" s="8"/>
-    </row>
-    <row r="106" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B106" s="8"/>
-      <c r="C106" s="8"/>
-      <c r="D106" s="8"/>
-      <c r="E106" s="8"/>
-      <c r="F106" s="8"/>
-      <c r="G106" s="8"/>
-      <c r="H106" s="8"/>
-      <c r="I106" s="8"/>
-      <c r="J106" s="8"/>
-      <c r="K106" s="8"/>
-      <c r="L106" s="8"/>
-      <c r="M106" s="8"/>
-    </row>
-    <row r="107" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B107" s="8"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="8"/>
-      <c r="E107" s="8"/>
-      <c r="F107" s="8"/>
-      <c r="G107" s="8"/>
-      <c r="H107" s="8"/>
-      <c r="I107" s="8"/>
-      <c r="J107" s="8"/>
-      <c r="K107" s="8"/>
-      <c r="L107" s="8"/>
-      <c r="M107" s="8"/>
-    </row>
-    <row r="108" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B108" s="8"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="8"/>
-      <c r="E108" s="8"/>
-      <c r="F108" s="8"/>
-      <c r="G108" s="8"/>
-      <c r="H108" s="8"/>
-      <c r="I108" s="8"/>
-      <c r="J108" s="8"/>
-      <c r="K108" s="8"/>
-      <c r="L108" s="8"/>
-      <c r="M108" s="8"/>
-    </row>
-    <row r="109" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B109" s="8"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="8"/>
-      <c r="E109" s="8"/>
-      <c r="F109" s="8"/>
-      <c r="G109" s="8"/>
-      <c r="H109" s="8"/>
-      <c r="I109" s="8"/>
-      <c r="J109" s="8"/>
-      <c r="K109" s="8"/>
-      <c r="L109" s="8"/>
-      <c r="M109" s="8"/>
-    </row>
-    <row r="110" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B110" s="8"/>
-      <c r="C110" s="8"/>
-      <c r="D110" s="8"/>
-      <c r="E110" s="8"/>
-      <c r="F110" s="8"/>
-      <c r="G110" s="8"/>
-      <c r="H110" s="8"/>
-      <c r="I110" s="8"/>
-      <c r="J110" s="8"/>
-      <c r="K110" s="8"/>
-      <c r="L110" s="8"/>
-      <c r="M110" s="8"/>
-    </row>
-    <row r="111" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B111" s="8"/>
-      <c r="C111" s="8"/>
-      <c r="D111" s="8"/>
-      <c r="E111" s="8"/>
-      <c r="F111" s="8"/>
-      <c r="G111" s="8"/>
-      <c r="H111" s="8"/>
-      <c r="I111" s="8"/>
-      <c r="J111" s="8"/>
-      <c r="K111" s="8"/>
-      <c r="L111" s="8"/>
-      <c r="M111" s="8"/>
-    </row>
-    <row r="112" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B112" s="8"/>
-      <c r="C112" s="8"/>
-      <c r="D112" s="8"/>
-      <c r="E112" s="8"/>
-      <c r="F112" s="8"/>
-      <c r="G112" s="8"/>
-      <c r="H112" s="8"/>
-      <c r="I112" s="8"/>
-      <c r="J112" s="8"/>
-      <c r="K112" s="8"/>
-      <c r="L112" s="8"/>
-      <c r="M112" s="8"/>
-    </row>
-    <row r="113" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B113" s="8"/>
-      <c r="C113" s="8"/>
-      <c r="D113" s="8"/>
-      <c r="E113" s="8"/>
-      <c r="F113" s="8"/>
-      <c r="G113" s="8"/>
-      <c r="H113" s="8"/>
-      <c r="I113" s="8"/>
-      <c r="J113" s="8"/>
-      <c r="K113" s="8"/>
-      <c r="L113" s="8"/>
-      <c r="M113" s="8"/>
-    </row>
-    <row r="114" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A80" s="1">
+        <v>79</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D80" s="8">
+        <v>12000</v>
+      </c>
+      <c r="E80" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F80" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G80" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H80" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="I80" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J80" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K80" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L80" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M80" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A81" s="1">
+        <v>80</v>
+      </c>
+      <c r="B81" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C81" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D81" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E81" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H81" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="I81" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J81" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K81" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L81" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="M81" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A82" s="1">
+        <v>81</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D82" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E82" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F82" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G82" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H82" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="I82" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J82" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K82" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="L82" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="M82" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A83" s="1">
+        <v>82</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D83" s="8">
+        <v>68000</v>
+      </c>
+      <c r="E83" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F83" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G83" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H83" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="I83" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J83" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K83" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="L83" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="M83" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A84" s="1">
+        <v>83</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D84" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E84" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F84" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G84" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H84" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="I84" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J84" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K84" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L84" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="M84" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A85" s="1">
+        <v>84</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D85" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G85" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H85" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="I85" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J85" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K85" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L85" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="M85" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A86" s="1">
+        <v>85</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D86" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E86" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F86" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H86" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="I86" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J86" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K86" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L86" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="M86" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" s="1">
+        <v>86</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D87" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H87" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J87" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K87" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L87" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="M87" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" s="1">
+        <v>87</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D88" s="8">
+        <v>56000</v>
+      </c>
+      <c r="E88" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F88" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G88" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H88" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="I88" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J88" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K88" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L88" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="M88" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" s="1">
+        <v>88</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D89" s="8">
+        <v>56000</v>
+      </c>
+      <c r="E89" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F89" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G89" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H89" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="I89" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J89" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K89" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L89" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="M89" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" s="1">
+        <v>89</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D90" s="8">
+        <v>54000</v>
+      </c>
+      <c r="E90" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F90" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G90" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H90" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I90" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J90" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K90" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L90" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="M90" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" s="1">
+        <v>90</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D91" s="8">
+        <v>54000</v>
+      </c>
+      <c r="E91" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F91" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G91" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H91" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="I91" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J91" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K91" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L91" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="M91" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" s="1">
+        <v>91</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D92" s="8">
+        <v>49000</v>
+      </c>
+      <c r="E92" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F92" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G92" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H92" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="I92" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J92" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K92" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L92" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="M92" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" s="1">
+        <v>92</v>
+      </c>
+      <c r="B93" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D93" s="8">
+        <v>49000</v>
+      </c>
+      <c r="E93" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F93" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G93" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H93" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="I93" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J93" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K93" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L93" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="M93" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" s="1">
+        <v>93</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D94" s="8">
+        <v>17000</v>
+      </c>
+      <c r="E94" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F94" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G94" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H94" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="I94" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J94" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K94" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L94" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M94" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" s="1">
+        <v>94</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D95" s="8">
+        <v>25000</v>
+      </c>
+      <c r="E95" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F95" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G95" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H95" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="I95" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J95" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K95" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L95" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M95" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" s="1">
+        <v>95</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D96" s="8">
+        <v>28000</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F96" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="G96" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H96" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="I96" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J96" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K96" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L96" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M96" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" s="1">
+        <v>96</v>
+      </c>
+      <c r="B97" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D97" s="8">
+        <v>12500</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F97" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G97" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H97" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="I97" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J97" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K97" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L97" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M97" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" s="1">
+        <v>97</v>
+      </c>
+      <c r="B98" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D98" s="8">
+        <v>55000</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F98" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G98" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H98" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="I98" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J98" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K98" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="L98" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M98" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A99" s="1">
+        <v>98</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C99" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D99" s="8">
+        <v>40000</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G99" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H99" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="I99" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J99" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K99" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L99" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="M99" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A100" s="1">
+        <v>99</v>
+      </c>
+      <c r="B100" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D100" s="8">
+        <v>22000</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F100" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G100" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H100" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="I100" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J100" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K100" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L100" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M100" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A101" s="1">
+        <v>100</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D101" s="8">
+        <v>22000</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F101" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G101" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H101" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="I101" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J101" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K101" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L101" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M101" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A102" s="1">
+        <v>101</v>
+      </c>
+      <c r="B102" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D102" s="8">
+        <v>22000</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F102" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G102" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H102" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="I102" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J102" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K102" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L102" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M102" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="103" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A103" s="1">
+        <v>102</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C103" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D103" s="8">
+        <v>22000</v>
+      </c>
+      <c r="E103" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F103" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G103" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H103" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="I103" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J103" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K103" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L103" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M103" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="104" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A104" s="1">
+        <v>103</v>
+      </c>
+      <c r="B104" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D104" s="8">
+        <v>25000</v>
+      </c>
+      <c r="E104" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F104" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G104" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="I104" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J104" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K104" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L104" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M104" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="105" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A105" s="1">
+        <v>104</v>
+      </c>
+      <c r="B105" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C105" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D105" s="8">
+        <v>25000</v>
+      </c>
+      <c r="E105" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F105" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G105" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H105" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="I105" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J105" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K105" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L105" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="M105" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="106" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A106" s="1">
+        <v>105</v>
+      </c>
+      <c r="B106" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D106" s="8">
+        <v>26000</v>
+      </c>
+      <c r="E106" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F106" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G106" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H106" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="I106" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J106" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K106" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L106" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="M106" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="107" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="1">
+        <v>106</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D107" s="8">
+        <v>26000</v>
+      </c>
+      <c r="E107" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F107" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="G107" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H107" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="I107" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J107" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K107" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="L107" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="M107" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="108" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A108" s="1">
+        <v>107</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C108" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D108" s="8">
+        <v>26000</v>
+      </c>
+      <c r="E108" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F108" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="G108" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H108" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="I108" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J108" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K108" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L108" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="M108" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="109" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A109" s="1">
+        <v>108</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D109" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E109" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F109" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G109" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H109" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="I109" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J109" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K109" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="L109" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="M109" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="1">
+        <v>109</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D110" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E110" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F110" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G110" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H110" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="I110" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J110" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K110" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L110" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="M110" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="111" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="1">
+        <v>110</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C111" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D111" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E111" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F111" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G111" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H111" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="I111" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J111" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K111" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L111" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="M111" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="112" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="1">
+        <v>111</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C112" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D112" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E112" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F112" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G112" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H112" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="I112" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J112" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K112" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L112" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="M112" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="1">
+        <v>112</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D113" s="8">
+        <v>80000</v>
+      </c>
+      <c r="E113" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F113" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G113" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H113" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="I113" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J113" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K113" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L113" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="M113" s="10">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B114" s="8"/>
       <c r="C114" s="8"/>
       <c r="D114" s="8"/>
@@ -4492,7 +5778,7 @@
       <c r="L114" s="8"/>
       <c r="M114" s="8"/>
     </row>
-    <row r="115" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B115" s="8"/>
       <c r="C115" s="8"/>
       <c r="D115" s="8"/>
@@ -4506,7 +5792,7 @@
       <c r="L115" s="8"/>
       <c r="M115" s="8"/>
     </row>
-    <row r="116" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B116" s="8"/>
       <c r="C116" s="8"/>
       <c r="D116" s="8"/>
@@ -4520,7 +5806,7 @@
       <c r="L116" s="8"/>
       <c r="M116" s="8"/>
     </row>
-    <row r="117" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B117" s="8"/>
       <c r="C117" s="8"/>
       <c r="D117" s="8"/>
@@ -4534,7 +5820,7 @@
       <c r="L117" s="8"/>
       <c r="M117" s="8"/>
     </row>
-    <row r="118" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B118" s="8"/>
       <c r="C118" s="8"/>
       <c r="D118" s="8"/>
@@ -4548,7 +5834,7 @@
       <c r="L118" s="8"/>
       <c r="M118" s="8"/>
     </row>
-    <row r="119" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B119" s="8"/>
       <c r="C119" s="8"/>
       <c r="D119" s="8"/>
@@ -4562,7 +5848,7 @@
       <c r="L119" s="8"/>
       <c r="M119" s="8"/>
     </row>
-    <row r="120" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B120" s="8"/>
       <c r="C120" s="8"/>
       <c r="D120" s="8"/>
@@ -4576,7 +5862,7 @@
       <c r="L120" s="8"/>
       <c r="M120" s="8"/>
     </row>
-    <row r="121" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B121" s="8"/>
       <c r="C121" s="8"/>
       <c r="D121" s="8"/>
@@ -4590,7 +5876,7 @@
       <c r="L121" s="8"/>
       <c r="M121" s="8"/>
     </row>
-    <row r="122" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B122" s="8"/>
       <c r="C122" s="8"/>
       <c r="D122" s="8"/>
@@ -4604,7 +5890,7 @@
       <c r="L122" s="8"/>
       <c r="M122" s="8"/>
     </row>
-    <row r="123" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B123" s="8"/>
       <c r="C123" s="8"/>
       <c r="D123" s="8"/>
@@ -4618,7 +5904,7 @@
       <c r="L123" s="8"/>
       <c r="M123" s="8"/>
     </row>
-    <row r="124" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B124" s="8"/>
       <c r="C124" s="8"/>
       <c r="D124" s="8"/>
@@ -4632,7 +5918,7 @@
       <c r="L124" s="8"/>
       <c r="M124" s="8"/>
     </row>
-    <row r="125" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B125" s="8"/>
       <c r="C125" s="8"/>
       <c r="D125" s="8"/>
@@ -4646,7 +5932,7 @@
       <c r="L125" s="8"/>
       <c r="M125" s="8"/>
     </row>
-    <row r="126" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B126" s="8"/>
       <c r="C126" s="8"/>
       <c r="D126" s="8"/>
@@ -4660,7 +5946,7 @@
       <c r="L126" s="8"/>
       <c r="M126" s="8"/>
     </row>
-    <row r="127" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B127" s="8"/>
       <c r="C127" s="8"/>
       <c r="D127" s="8"/>
@@ -4674,7 +5960,7 @@
       <c r="L127" s="8"/>
       <c r="M127" s="8"/>
     </row>
-    <row r="128" spans="2:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B128" s="8"/>
       <c r="C128" s="8"/>
       <c r="D128" s="8"/>
@@ -4997,6 +6283,27 @@
     <hyperlink ref="H8" r:id="rId67" xr:uid="{BC392C16-44E5-0247-9603-E28D1664E0BC}"/>
     <hyperlink ref="H7" r:id="rId68" xr:uid="{BEC9B471-A176-CF47-9FCA-E2FA242AA85A}"/>
     <hyperlink ref="H5" r:id="rId69" xr:uid="{97C5CAB9-0FD9-2E44-87D6-AEDA82ABBA70}"/>
+    <hyperlink ref="H74" r:id="rId70" xr:uid="{355C4807-A326-4049-8B18-EC4BCCEA6771}"/>
+    <hyperlink ref="H75" r:id="rId71" xr:uid="{B4C967E2-25EB-224A-9375-D5553A65BDEC}"/>
+    <hyperlink ref="H76" r:id="rId72" xr:uid="{2047E8E9-D291-0147-A1AE-D2247FC8E7B7}"/>
+    <hyperlink ref="H77" r:id="rId73" xr:uid="{57F780E1-013A-B44B-A78A-8E13971240FA}"/>
+    <hyperlink ref="H78" r:id="rId74" xr:uid="{1FD5469F-F1A8-C74A-AF18-780AB15ADA48}"/>
+    <hyperlink ref="H79" r:id="rId75" xr:uid="{FDA055D6-AEAC-A848-86A9-941A9B5E6677}"/>
+    <hyperlink ref="H80" r:id="rId76" xr:uid="{7977804C-3A1F-EB43-AC0B-2A16CC437FED}"/>
+    <hyperlink ref="H100" r:id="rId77" xr:uid="{F6A44307-984E-9E4A-BB29-2096E232D52E}"/>
+    <hyperlink ref="H101" r:id="rId78" xr:uid="{BBB7AEA8-A3E7-2540-9D64-555CF198F0AE}"/>
+    <hyperlink ref="H102" r:id="rId79" xr:uid="{31638D57-F9A1-8440-8AAA-FB7EC3275284}"/>
+    <hyperlink ref="H103" r:id="rId80" xr:uid="{4D67B34A-C716-1048-B21D-FD65FA1FC86A}"/>
+    <hyperlink ref="H104" r:id="rId81" xr:uid="{4F9974E9-281F-324B-B2B6-DB64B7988717}"/>
+    <hyperlink ref="H105" r:id="rId82" xr:uid="{790876C7-43B0-1641-9648-4DA5B66C4E6A}"/>
+    <hyperlink ref="H106" r:id="rId83" xr:uid="{D645509F-DAD4-1B48-AE27-1756FF478CC6}"/>
+    <hyperlink ref="H107" r:id="rId84" xr:uid="{329E350C-1CF8-5C45-95C6-4C3E372F91C2}"/>
+    <hyperlink ref="H108" r:id="rId85" xr:uid="{469EFC21-E4CF-EA44-97D3-E3BC30FBA948}"/>
+    <hyperlink ref="H109" r:id="rId86" xr:uid="{6F4FFC68-88CD-BF45-B17F-2DF461BC021E}"/>
+    <hyperlink ref="H110" r:id="rId87" xr:uid="{234BD536-ADCB-C642-AC40-BC68C8BC75ED}"/>
+    <hyperlink ref="H111" r:id="rId88" xr:uid="{0F913E7E-15FD-6443-9176-9E98916E93F7}"/>
+    <hyperlink ref="H112" r:id="rId89" xr:uid="{7560FF78-E43C-8F41-8F50-98A5F3538B83}"/>
+    <hyperlink ref="H113" r:id="rId90" xr:uid="{97F9E249-BE09-A44A-9460-BA5D56C0AF7D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync products.xlsx and regenerate cards
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a/ЛСсайт/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0D2ACE-2770-6F43-9720-9CD3B078663E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349938B9-A317-C343-A87F-1BFEE5D34AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -610,45 +610,27 @@
     <t>Сумка Chanel</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915641/tg-products/stkyhzzdkuh1cgimaizl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915643/tg-products/tzko9pcwffbbwbbufkfv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915648/tg-products/uf0pp82dkddefxuqld1s.jpg</t>
-  </si>
-  <si>
     <t>23х14х6 см</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915701/tg-products/bvup6c9kmi4zlzidrgyq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915713/tg-products/qmmjhrb4i7hnshqgbiyb.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915721/tg-products/rqlei70guawavf6fhzjo.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915768/tg-products/xalpgyleamdxmb1oyzq9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915771/tg-products/fumo4n1kyawnlcva1nif.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915786/tg-products/c53oo1tsfepwatxfoqdc.jpg</t>
   </si>
   <si>
     <t>17х14х8 см</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915974/tg-products/okpiwinqf4jcsf7nr3hf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915983/tg-products/hqs27dixwbs9zfsletjk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915992/tg-products/klvb2yk28squrw4eqcoe.jpg</t>
-  </si>
-  <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916026/tg-products/v3bzscftxxtfkok5cdaf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916040/tg-products/cul4h6zea2sonxd1lgxf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916055/tg-products/mffin77lcud3f2op2cyd.jpg</t>
-  </si>
-  <si>
     <t>22х20х13 см</t>
   </si>
   <si>
     <t>Материал ткань</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916102/tg-products/fnje0ov6zeyrfokmxdks.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916113/tg-products/cgpw0axs1slqut7jrnrk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916132/tg-products/tbbqejtlrdnzpynr0nws.jpg</t>
-  </si>
-  <si>
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916086/tg-products/sddmxitn3mxmgthy2cp1.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916093/tg-products/wxfglpoym9jkav8kz9kf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916138/tg-products/qlzplygyrsjonuc6kiqk.jpg</t>
   </si>
   <si>
     <t>Рюкзак Miumiu</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916432/tg-products/l1wohpgzi9o8rnu80flv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916436/tg-products/mrmuffh9c6uvbhg9s7rk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916445/tg-products/ilk8cs62va6xydzdmstw.jpg</t>
-  </si>
-  <si>
     <t>30х25х13 см</t>
   </si>
   <si>
@@ -670,15 +652,9 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916555/tg-products/pwqnaichbddjbn9oapdd.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916564/tg-products/znxg24dqz9iogwltnsg8.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916590/tg-products/ot81lsalffufeiq8rks1.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916922/tg-products/eootmyjtcnsi4yr4m62z.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916929/tg-products/fotezp5mzile8hxif7dl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916940/tg-products/ghkrsbfqxkpdjudellin.jpg</t>
-  </si>
-  <si>
     <t>33х19х5 см</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916978/tg-products/l1haqfjdigfv4gznyeea.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg</t>
-  </si>
-  <si>
     <t>серый</t>
   </si>
   <si>
@@ -785,6 +761,30 @@
   </si>
   <si>
     <t>Louis Vuitton</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915648/tg-products/uf0pp82dkddefxuqld1s.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915641/tg-products/stkyhzzdkuh1cgimaizl.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915643/tg-products/tzko9pcwffbbwbbufkfv.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915721/tg-products/rqlei70guawavf6fhzjo.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915701/tg-products/bvup6c9kmi4zlzidrgyq.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915713/tg-products/qmmjhrb4i7hnshqgbiyb.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915983/tg-products/hqs27dixwbs9zfsletjk.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915992/tg-products/klvb2yk28squrw4eqcoe.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915974/tg-products/okpiwinqf4jcsf7nr3hf.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916055/tg-products/mffin77lcud3f2op2cyd.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916026/tg-products/v3bzscftxxtfkok5cdaf.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916040/tg-products/cul4h6zea2sonxd1lgxf.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916132/tg-products/tbbqejtlrdnzpynr0nws.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916102/tg-products/fnje0ov6zeyrfokmxdks.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916113/tg-products/cgpw0axs1slqut7jrnrk.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916445/tg-products/ilk8cs62va6xydzdmstw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916432/tg-products/l1wohpgzi9o8rnu80flv.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916436/tg-products/mrmuffh9c6uvbhg9s7rk.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916978/tg-products/l1haqfjdigfv4gznyeea.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916922/tg-products/eootmyjtcnsi4yr4m62z.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916929/tg-products/fotezp5mzile8hxif7dl.jpg</t>
   </si>
 </sst>
 </file>
@@ -4434,7 +4434,7 @@
         <v>70</v>
       </c>
       <c r="H81" s="8" t="s">
-        <v>196</v>
+        <v>247</v>
       </c>
       <c r="I81" s="8" t="s">
         <v>20</v>
@@ -4446,7 +4446,7 @@
         <v>87</v>
       </c>
       <c r="L81" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M81" s="10">
         <v>46100</v>
@@ -4475,7 +4475,7 @@
         <v>70</v>
       </c>
       <c r="H82" s="8" t="s">
-        <v>198</v>
+        <v>248</v>
       </c>
       <c r="I82" s="8" t="s">
         <v>20</v>
@@ -4484,10 +4484,10 @@
         <v>21</v>
       </c>
       <c r="K82" s="8" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="L82" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M82" s="10">
         <v>46100</v>
@@ -4516,7 +4516,7 @@
         <v>70</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I83" s="8" t="s">
         <v>20</v>
@@ -4528,7 +4528,7 @@
         <v>130</v>
       </c>
       <c r="L83" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="M83" s="10">
         <v>46100</v>
@@ -4557,7 +4557,7 @@
         <v>70</v>
       </c>
       <c r="H84" s="8" t="s">
-        <v>201</v>
+        <v>249</v>
       </c>
       <c r="I84" s="8" t="s">
         <v>20</v>
@@ -4569,7 +4569,7 @@
         <v>30</v>
       </c>
       <c r="L84" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M84" s="10">
         <v>46100</v>
@@ -4598,7 +4598,7 @@
         <v>70</v>
       </c>
       <c r="H85" s="8" t="s">
-        <v>202</v>
+        <v>250</v>
       </c>
       <c r="I85" s="8" t="s">
         <v>20</v>
@@ -4610,7 +4610,7 @@
         <v>85</v>
       </c>
       <c r="L85" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="M85" s="10">
         <v>46100</v>
@@ -4633,13 +4633,13 @@
         <v>16</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G86" s="8" t="s">
         <v>70</v>
       </c>
       <c r="H86" s="8" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="I86" s="8" t="s">
         <v>20</v>
@@ -4651,7 +4651,7 @@
         <v>41</v>
       </c>
       <c r="L86" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="M86" s="10">
         <v>46100</v>
@@ -4680,7 +4680,7 @@
         <v>70</v>
       </c>
       <c r="H87" s="8" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="I87" s="8" t="s">
         <v>20</v>
@@ -4692,7 +4692,7 @@
         <v>30</v>
       </c>
       <c r="L87" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="M87" s="10">
         <v>46100</v>
@@ -4703,7 +4703,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>64</v>
@@ -4721,7 +4721,7 @@
         <v>70</v>
       </c>
       <c r="H88" s="8" t="s">
-        <v>208</v>
+        <v>252</v>
       </c>
       <c r="I88" s="8" t="s">
         <v>20</v>
@@ -4733,7 +4733,7 @@
         <v>87</v>
       </c>
       <c r="L88" s="8" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="M88" s="10">
         <v>46100</v>
@@ -4744,7 +4744,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>64</v>
@@ -4756,13 +4756,13 @@
         <v>16</v>
       </c>
       <c r="F89" s="9" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G89" s="8" t="s">
         <v>70</v>
       </c>
       <c r="H89" s="8" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="I89" s="8" t="s">
         <v>20</v>
@@ -4774,7 +4774,7 @@
         <v>87</v>
       </c>
       <c r="L89" s="8" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="M89" s="10">
         <v>46100</v>
@@ -4785,7 +4785,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>64</v>
@@ -4803,7 +4803,7 @@
         <v>70</v>
       </c>
       <c r="H90" s="8" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="I90" s="8" t="s">
         <v>20</v>
@@ -4815,7 +4815,7 @@
         <v>85</v>
       </c>
       <c r="L90" s="8" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="M90" s="10">
         <v>46100</v>
@@ -4826,7 +4826,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>64</v>
@@ -4844,7 +4844,7 @@
         <v>70</v>
       </c>
       <c r="H91" s="8" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="I91" s="8" t="s">
         <v>20</v>
@@ -4856,7 +4856,7 @@
         <v>87</v>
       </c>
       <c r="L91" s="8" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="M91" s="10">
         <v>46100</v>
@@ -4867,7 +4867,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>64</v>
@@ -4885,7 +4885,7 @@
         <v>70</v>
       </c>
       <c r="H92" s="8" t="s">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="I92" s="8" t="s">
         <v>20</v>
@@ -4897,7 +4897,7 @@
         <v>85</v>
       </c>
       <c r="L92" s="8" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="M92" s="10">
         <v>46100</v>
@@ -4908,7 +4908,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>64</v>
@@ -4926,7 +4926,7 @@
         <v>70</v>
       </c>
       <c r="H93" s="8" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="I93" s="8" t="s">
         <v>20</v>
@@ -4938,7 +4938,7 @@
         <v>87</v>
       </c>
       <c r="L93" s="8" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="M93" s="10">
         <v>46100</v>
@@ -4949,10 +4949,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="D94" s="8">
         <v>17000</v>
@@ -4967,7 +4967,7 @@
         <v>18</v>
       </c>
       <c r="H94" s="8" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="I94" s="8" t="s">
         <v>20</v>
@@ -4990,10 +4990,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="D95" s="8">
         <v>25000</v>
@@ -5008,7 +5008,7 @@
         <v>18</v>
       </c>
       <c r="H95" s="8" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="I95" s="8" t="s">
         <v>20</v>
@@ -5031,7 +5031,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C96" s="8" t="s">
         <v>89</v>
@@ -5043,13 +5043,13 @@
         <v>16</v>
       </c>
       <c r="F96" s="9" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="G96" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H96" s="8" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="I96" s="8" t="s">
         <v>20</v>
@@ -5072,7 +5072,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>60</v>
@@ -5090,7 +5090,7 @@
         <v>18</v>
       </c>
       <c r="H97" s="8" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="I97" s="8" t="s">
         <v>20</v>
@@ -5131,7 +5131,7 @@
         <v>18</v>
       </c>
       <c r="H98" s="8" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="I98" s="8" t="s">
         <v>20</v>
@@ -5154,10 +5154,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="D99" s="8">
         <v>40000</v>
@@ -5172,7 +5172,7 @@
         <v>18</v>
       </c>
       <c r="H99" s="8" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="I99" s="8" t="s">
         <v>20</v>
@@ -5195,7 +5195,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>141</v>
@@ -5213,7 +5213,7 @@
         <v>90</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="I100" s="8" t="s">
         <v>20</v>
@@ -5236,7 +5236,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>141</v>
@@ -5254,7 +5254,7 @@
         <v>90</v>
       </c>
       <c r="H101" s="11" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="I101" s="8" t="s">
         <v>20</v>
@@ -5277,7 +5277,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>141</v>
@@ -5295,7 +5295,7 @@
         <v>90</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="I102" s="8" t="s">
         <v>20</v>
@@ -5318,7 +5318,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C103" s="8" t="s">
         <v>141</v>
@@ -5336,7 +5336,7 @@
         <v>90</v>
       </c>
       <c r="H103" s="11" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="I103" s="8" t="s">
         <v>20</v>
@@ -5359,7 +5359,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C104" s="8" t="s">
         <v>48</v>
@@ -5377,7 +5377,7 @@
         <v>90</v>
       </c>
       <c r="H104" s="11" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="I104" s="8" t="s">
         <v>20</v>
@@ -5400,7 +5400,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>48</v>
@@ -5418,7 +5418,7 @@
         <v>90</v>
       </c>
       <c r="H105" s="11" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="I105" s="8" t="s">
         <v>20</v>
@@ -5441,7 +5441,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="C106" s="8" t="s">
         <v>48</v>
@@ -5459,7 +5459,7 @@
         <v>90</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="I106" s="8" t="s">
         <v>20</v>
@@ -5482,7 +5482,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C107" s="8" t="s">
         <v>48</v>
@@ -5494,13 +5494,13 @@
         <v>16</v>
       </c>
       <c r="F107" s="9" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G107" s="8" t="s">
         <v>90</v>
       </c>
       <c r="H107" s="11" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="I107" s="8" t="s">
         <v>20</v>
@@ -5523,7 +5523,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>48</v>
@@ -5535,13 +5535,13 @@
         <v>16</v>
       </c>
       <c r="F108" s="9" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G108" s="8" t="s">
         <v>90</v>
       </c>
       <c r="H108" s="11" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="I108" s="8" t="s">
         <v>20</v>
@@ -5582,7 +5582,7 @@
         <v>70</v>
       </c>
       <c r="H109" s="11" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="I109" s="8" t="s">
         <v>20</v>
@@ -5594,7 +5594,7 @@
         <v>130</v>
       </c>
       <c r="L109" s="8" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="M109" s="10">
         <v>46100</v>
@@ -5623,7 +5623,7 @@
         <v>70</v>
       </c>
       <c r="H110" s="11" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="I110" s="8" t="s">
         <v>20</v>
@@ -5635,7 +5635,7 @@
         <v>85</v>
       </c>
       <c r="L110" s="8" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="M110" s="10">
         <v>46100</v>
@@ -5664,7 +5664,7 @@
         <v>70</v>
       </c>
       <c r="H111" s="11" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="I111" s="8" t="s">
         <v>20</v>
@@ -5676,7 +5676,7 @@
         <v>96</v>
       </c>
       <c r="L111" s="8" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="M111" s="10">
         <v>46100</v>
@@ -5705,7 +5705,7 @@
         <v>70</v>
       </c>
       <c r="H112" s="11" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="I112" s="8" t="s">
         <v>20</v>
@@ -5717,7 +5717,7 @@
         <v>30</v>
       </c>
       <c r="L112" s="8" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="M112" s="10">
         <v>46100</v>
@@ -5746,7 +5746,7 @@
         <v>70</v>
       </c>
       <c r="H113" s="11" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="I113" s="8" t="s">
         <v>20</v>
@@ -5758,7 +5758,7 @@
         <v>26</v>
       </c>
       <c r="L113" s="8" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="M113" s="10">
         <v>46100</v>

</xml_diff>

<commit_message>
Sync products from products.xlsx
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a/ЛСсайт/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349938B9-A317-C343-A87F-1BFEE5D34AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCBA49C-6C8A-2249-AAC7-D26080679A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="254">
   <si>
     <t>id</t>
   </si>
@@ -604,9 +604,6 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915010/tg-products/akcys7bv9vxcmdeppsuk.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773915133/tg-products/qq6oo9af9mwumggnc1qz.jpg</t>
-  </si>
-  <si>
     <t>Сумка Chanel</t>
   </si>
   <si>
@@ -661,15 +658,9 @@
     <t>Топ Fendi</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933748/tg-products/xdb2jkfqk6wesecqdolt.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933749/tg-products/mgcrk3utqbezfs4ixztw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933756/tg-products/yiu9q66cs6mwcfahauri.jpg</t>
-  </si>
-  <si>
     <t>Рубашка Fendi</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933794/tg-products/bdl0j9ioh5mayldrjmfw.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933795/tg-products/enspkgek73kduyxzd0e9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933796/tg-products/hvt9ykb7wv9vwn2fegto.jpg</t>
-  </si>
-  <si>
     <t>Свитер Hermes</t>
   </si>
   <si>
@@ -685,15 +676,9 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933876/tg-products/fuldr5oxwjl4ofjtyvb5.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933881/tg-products/zxsbuqp1zi6fmudrcrge.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933882/tg-products/ibvz2vhk5zjttfjncoju.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933931/tg-products/y3preqgf4yrmzvjiabuh.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933932/tg-products/ko7czxgykv0usognjmff.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933933/tg-products/bnlf6iyyg9u6mlqciplj.jpg</t>
-  </si>
-  <si>
     <t>Платье Louis Vuitton</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773934457/tg-products/ltj8m2vwgmhol94h9ood.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940115/tg-products/zynb4me8jy8291jyhwo9.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773940116/tg-products/guma9ms2hjqdeypzy08k.jpg</t>
-  </si>
-  <si>
     <t>Лоферы Loro Piana</t>
   </si>
   <si>
@@ -784,7 +769,19 @@
     <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916978/tg-products/l1haqfjdigfv4gznyeea.jpg</t>
   </si>
   <si>
-    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773917006/tg-products/dtnurtt0jdklt6jjovtn.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916922/tg-products/eootmyjtcnsi4yr4m62z.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773916929/tg-products/fotezp5mzile8hxif7dl.jpg</t>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933749/tg-products/mgcrk3utqbezfs4ixztw.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933796/tg-products/hvt9ykb7wv9vwn2fegto.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773934457/tg-products/ltj8m2vwgmhol94h9ood.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933932/tg-products/ko7czxgykv0usognjmff.jpg, https://res.cloudinary.com/dlexrnrhe/image/upload/v1773933933/tg-products/bnlf6iyyg9u6mlqciplj.jpg</t>
+  </si>
+  <si>
+    <t>₽+E116</t>
   </si>
 </sst>
 </file>
@@ -4375,25 +4372,25 @@
         <v>79</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>13</v>
+        <v>194</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="D80" s="8">
-        <v>12000</v>
+        <v>80000</v>
       </c>
       <c r="E80" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F80" s="9" t="s">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="G80" s="8" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="H80" s="11" t="s">
-        <v>194</v>
+        <v>237</v>
       </c>
       <c r="I80" s="8" t="s">
         <v>20</v>
@@ -4405,7 +4402,7 @@
         <v>30</v>
       </c>
       <c r="L80" s="8" t="s">
-        <v>115</v>
+        <v>234</v>
       </c>
       <c r="M80" s="10">
         <v>46100</v>
@@ -4416,7 +4413,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>48</v>
@@ -4434,7 +4431,7 @@
         <v>70</v>
       </c>
       <c r="H81" s="8" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="I81" s="8" t="s">
         <v>20</v>
@@ -4446,7 +4443,7 @@
         <v>87</v>
       </c>
       <c r="L81" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M81" s="10">
         <v>46100</v>
@@ -4457,7 +4454,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>48</v>
@@ -4475,7 +4472,7 @@
         <v>70</v>
       </c>
       <c r="H82" s="8" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="I82" s="8" t="s">
         <v>20</v>
@@ -4484,10 +4481,10 @@
         <v>21</v>
       </c>
       <c r="K82" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L82" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M82" s="10">
         <v>46100</v>
@@ -4498,7 +4495,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>48</v>
@@ -4516,7 +4513,7 @@
         <v>70</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I83" s="8" t="s">
         <v>20</v>
@@ -4528,7 +4525,7 @@
         <v>130</v>
       </c>
       <c r="L83" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="M83" s="10">
         <v>46100</v>
@@ -4539,7 +4536,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>48</v>
@@ -4557,7 +4554,7 @@
         <v>70</v>
       </c>
       <c r="H84" s="8" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="I84" s="8" t="s">
         <v>20</v>
@@ -4569,7 +4566,7 @@
         <v>30</v>
       </c>
       <c r="L84" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M84" s="10">
         <v>46100</v>
@@ -4580,7 +4577,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>48</v>
@@ -4598,7 +4595,7 @@
         <v>70</v>
       </c>
       <c r="H85" s="8" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="I85" s="8" t="s">
         <v>20</v>
@@ -4610,7 +4607,7 @@
         <v>85</v>
       </c>
       <c r="L85" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M85" s="10">
         <v>46100</v>
@@ -4621,7 +4618,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>48</v>
@@ -4633,13 +4630,13 @@
         <v>16</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G86" s="8" t="s">
         <v>70</v>
       </c>
       <c r="H86" s="8" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I86" s="8" t="s">
         <v>20</v>
@@ -4651,7 +4648,7 @@
         <v>41</v>
       </c>
       <c r="L86" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M86" s="10">
         <v>46100</v>
@@ -4662,7 +4659,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>48</v>
@@ -4680,7 +4677,7 @@
         <v>70</v>
       </c>
       <c r="H87" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I87" s="8" t="s">
         <v>20</v>
@@ -4692,7 +4689,7 @@
         <v>30</v>
       </c>
       <c r="L87" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M87" s="10">
         <v>46100</v>
@@ -4703,7 +4700,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>64</v>
@@ -4721,7 +4718,7 @@
         <v>70</v>
       </c>
       <c r="H88" s="8" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="I88" s="8" t="s">
         <v>20</v>
@@ -4733,7 +4730,7 @@
         <v>87</v>
       </c>
       <c r="L88" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M88" s="10">
         <v>46100</v>
@@ -4744,7 +4741,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>64</v>
@@ -4756,13 +4753,13 @@
         <v>16</v>
       </c>
       <c r="F89" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G89" s="8" t="s">
         <v>70</v>
       </c>
       <c r="H89" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I89" s="8" t="s">
         <v>20</v>
@@ -4774,7 +4771,7 @@
         <v>87</v>
       </c>
       <c r="L89" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M89" s="10">
         <v>46100</v>
@@ -4785,7 +4782,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>64</v>
@@ -4803,7 +4800,7 @@
         <v>70</v>
       </c>
       <c r="H90" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I90" s="8" t="s">
         <v>20</v>
@@ -4815,7 +4812,7 @@
         <v>85</v>
       </c>
       <c r="L90" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M90" s="10">
         <v>46100</v>
@@ -4826,7 +4823,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>64</v>
@@ -4844,7 +4841,7 @@
         <v>70</v>
       </c>
       <c r="H91" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I91" s="8" t="s">
         <v>20</v>
@@ -4856,7 +4853,7 @@
         <v>87</v>
       </c>
       <c r="L91" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M91" s="10">
         <v>46100</v>
@@ -4867,13 +4864,13 @@
         <v>91</v>
       </c>
       <c r="B92" s="8" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="D92" s="8">
-        <v>49000</v>
+        <v>80000</v>
       </c>
       <c r="E92" s="9" t="s">
         <v>16</v>
@@ -4884,8 +4881,8 @@
       <c r="G92" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="H92" s="8" t="s">
-        <v>254</v>
+      <c r="H92" s="11" t="s">
+        <v>238</v>
       </c>
       <c r="I92" s="8" t="s">
         <v>20</v>
@@ -4894,10 +4891,10 @@
         <v>21</v>
       </c>
       <c r="K92" s="8" t="s">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="L92" s="8" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="M92" s="10">
         <v>46100</v>
@@ -4908,7 +4905,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>64</v>
@@ -4926,7 +4923,7 @@
         <v>70</v>
       </c>
       <c r="H93" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="I93" s="8" t="s">
         <v>20</v>
@@ -4938,7 +4935,7 @@
         <v>87</v>
       </c>
       <c r="L93" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M93" s="10">
         <v>46100</v>
@@ -4949,16 +4946,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D94" s="8">
         <v>17000</v>
       </c>
       <c r="E94" s="9" t="s">
-        <v>16</v>
+        <v>253</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>17</v>
@@ -4966,8 +4963,8 @@
       <c r="G94" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H94" s="8" t="s">
-        <v>213</v>
+      <c r="H94" s="11" t="s">
+        <v>249</v>
       </c>
       <c r="I94" s="8" t="s">
         <v>20</v>
@@ -4990,10 +4987,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D95" s="8">
         <v>25000</v>
@@ -5007,8 +5004,8 @@
       <c r="G95" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H95" s="8" t="s">
-        <v>215</v>
+      <c r="H95" s="11" t="s">
+        <v>250</v>
       </c>
       <c r="I95" s="8" t="s">
         <v>20</v>
@@ -5031,7 +5028,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C96" s="8" t="s">
         <v>89</v>
@@ -5043,13 +5040,13 @@
         <v>16</v>
       </c>
       <c r="F96" s="9" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="G96" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H96" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="I96" s="8" t="s">
         <v>20</v>
@@ -5072,7 +5069,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>60</v>
@@ -5090,7 +5087,7 @@
         <v>18</v>
       </c>
       <c r="H97" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I97" s="8" t="s">
         <v>20</v>
@@ -5131,7 +5128,7 @@
         <v>18</v>
       </c>
       <c r="H98" s="8" t="s">
-        <v>221</v>
+        <v>252</v>
       </c>
       <c r="I98" s="8" t="s">
         <v>20</v>
@@ -5154,10 +5151,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D99" s="8">
         <v>40000</v>
@@ -5171,8 +5168,8 @@
       <c r="G99" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H99" s="8" t="s">
-        <v>223</v>
+      <c r="H99" s="11" t="s">
+        <v>251</v>
       </c>
       <c r="I99" s="8" t="s">
         <v>20</v>
@@ -5195,7 +5192,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>141</v>
@@ -5213,7 +5210,7 @@
         <v>90</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="I100" s="8" t="s">
         <v>20</v>
@@ -5236,7 +5233,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>141</v>
@@ -5254,7 +5251,7 @@
         <v>90</v>
       </c>
       <c r="H101" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="I101" s="8" t="s">
         <v>20</v>
@@ -5277,7 +5274,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>141</v>
@@ -5295,7 +5292,7 @@
         <v>90</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="I102" s="8" t="s">
         <v>20</v>
@@ -5318,7 +5315,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C103" s="8" t="s">
         <v>141</v>
@@ -5336,7 +5333,7 @@
         <v>90</v>
       </c>
       <c r="H103" s="11" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="I103" s="8" t="s">
         <v>20</v>
@@ -5359,7 +5356,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="8" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C104" s="8" t="s">
         <v>48</v>
@@ -5377,7 +5374,7 @@
         <v>90</v>
       </c>
       <c r="H104" s="11" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="I104" s="8" t="s">
         <v>20</v>
@@ -5400,7 +5397,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>48</v>
@@ -5418,7 +5415,7 @@
         <v>90</v>
       </c>
       <c r="H105" s="11" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="I105" s="8" t="s">
         <v>20</v>
@@ -5441,7 +5438,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="8" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C106" s="8" t="s">
         <v>48</v>
@@ -5459,7 +5456,7 @@
         <v>90</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="I106" s="8" t="s">
         <v>20</v>
@@ -5482,7 +5479,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C107" s="8" t="s">
         <v>48</v>
@@ -5494,13 +5491,13 @@
         <v>16</v>
       </c>
       <c r="F107" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="G107" s="8" t="s">
         <v>90</v>
       </c>
       <c r="H107" s="11" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="I107" s="8" t="s">
         <v>20</v>
@@ -5523,7 +5520,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="8" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>48</v>
@@ -5535,13 +5532,13 @@
         <v>16</v>
       </c>
       <c r="F108" s="9" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="G108" s="8" t="s">
         <v>90</v>
       </c>
       <c r="H108" s="11" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="I108" s="8" t="s">
         <v>20</v>
@@ -5564,7 +5561,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C109" s="8" t="s">
         <v>48</v>
@@ -5582,7 +5579,7 @@
         <v>70</v>
       </c>
       <c r="H109" s="11" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="I109" s="8" t="s">
         <v>20</v>
@@ -5594,7 +5591,7 @@
         <v>130</v>
       </c>
       <c r="L109" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="M109" s="10">
         <v>46100</v>
@@ -5605,7 +5602,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C110" s="8" t="s">
         <v>48</v>
@@ -5623,7 +5620,7 @@
         <v>70</v>
       </c>
       <c r="H110" s="11" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="I110" s="8" t="s">
         <v>20</v>
@@ -5635,7 +5632,7 @@
         <v>85</v>
       </c>
       <c r="L110" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="M110" s="10">
         <v>46100</v>
@@ -5646,7 +5643,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>48</v>
@@ -5664,7 +5661,7 @@
         <v>70</v>
       </c>
       <c r="H111" s="11" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="I111" s="8" t="s">
         <v>20</v>
@@ -5676,93 +5673,41 @@
         <v>96</v>
       </c>
       <c r="L111" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="M111" s="10">
         <v>46100</v>
       </c>
     </row>
     <row r="112" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A112" s="1">
-        <v>111</v>
-      </c>
-      <c r="B112" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C112" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D112" s="8">
-        <v>80000</v>
-      </c>
-      <c r="E112" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F112" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="G112" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="H112" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="I112" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J112" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K112" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="L112" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="M112" s="10">
-        <v>46100</v>
-      </c>
+      <c r="A112" s="1"/>
+      <c r="B112" s="8"/>
+      <c r="C112" s="8"/>
+      <c r="D112" s="8"/>
+      <c r="E112" s="9"/>
+      <c r="F112" s="9"/>
+      <c r="G112" s="8"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="8"/>
+      <c r="J112" s="8"/>
+      <c r="K112" s="8"/>
+      <c r="L112" s="8"/>
+      <c r="M112" s="10"/>
     </row>
     <row r="113" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A113" s="1">
-        <v>112</v>
-      </c>
-      <c r="B113" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C113" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D113" s="8">
-        <v>80000</v>
-      </c>
-      <c r="E113" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F113" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="G113" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="H113" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="I113" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J113" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K113" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="L113" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="M113" s="10">
-        <v>46100</v>
-      </c>
+      <c r="A113" s="1"/>
+      <c r="B113" s="8"/>
+      <c r="C113" s="8"/>
+      <c r="D113" s="8"/>
+      <c r="E113" s="9"/>
+      <c r="F113" s="9"/>
+      <c r="G113" s="8"/>
+      <c r="H113" s="11"/>
+      <c r="I113" s="8"/>
+      <c r="J113" s="8"/>
+      <c r="K113" s="8"/>
+      <c r="L113" s="8"/>
+      <c r="M113" s="10"/>
     </row>
     <row r="114" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B114" s="8"/>
@@ -6289,21 +6234,23 @@
     <hyperlink ref="H77" r:id="rId73" xr:uid="{57F780E1-013A-B44B-A78A-8E13971240FA}"/>
     <hyperlink ref="H78" r:id="rId74" xr:uid="{1FD5469F-F1A8-C74A-AF18-780AB15ADA48}"/>
     <hyperlink ref="H79" r:id="rId75" xr:uid="{FDA055D6-AEAC-A848-86A9-941A9B5E6677}"/>
-    <hyperlink ref="H80" r:id="rId76" xr:uid="{7977804C-3A1F-EB43-AC0B-2A16CC437FED}"/>
-    <hyperlink ref="H100" r:id="rId77" xr:uid="{F6A44307-984E-9E4A-BB29-2096E232D52E}"/>
-    <hyperlink ref="H101" r:id="rId78" xr:uid="{BBB7AEA8-A3E7-2540-9D64-555CF198F0AE}"/>
-    <hyperlink ref="H102" r:id="rId79" xr:uid="{31638D57-F9A1-8440-8AAA-FB7EC3275284}"/>
-    <hyperlink ref="H103" r:id="rId80" xr:uid="{4D67B34A-C716-1048-B21D-FD65FA1FC86A}"/>
-    <hyperlink ref="H104" r:id="rId81" xr:uid="{4F9974E9-281F-324B-B2B6-DB64B7988717}"/>
-    <hyperlink ref="H105" r:id="rId82" xr:uid="{790876C7-43B0-1641-9648-4DA5B66C4E6A}"/>
-    <hyperlink ref="H106" r:id="rId83" xr:uid="{D645509F-DAD4-1B48-AE27-1756FF478CC6}"/>
-    <hyperlink ref="H107" r:id="rId84" xr:uid="{329E350C-1CF8-5C45-95C6-4C3E372F91C2}"/>
-    <hyperlink ref="H108" r:id="rId85" xr:uid="{469EFC21-E4CF-EA44-97D3-E3BC30FBA948}"/>
-    <hyperlink ref="H109" r:id="rId86" xr:uid="{6F4FFC68-88CD-BF45-B17F-2DF461BC021E}"/>
-    <hyperlink ref="H110" r:id="rId87" xr:uid="{234BD536-ADCB-C642-AC40-BC68C8BC75ED}"/>
-    <hyperlink ref="H111" r:id="rId88" xr:uid="{0F913E7E-15FD-6443-9176-9E98916E93F7}"/>
-    <hyperlink ref="H112" r:id="rId89" xr:uid="{7560FF78-E43C-8F41-8F50-98A5F3538B83}"/>
-    <hyperlink ref="H113" r:id="rId90" xr:uid="{97F9E249-BE09-A44A-9460-BA5D56C0AF7D}"/>
+    <hyperlink ref="H100" r:id="rId76" xr:uid="{F6A44307-984E-9E4A-BB29-2096E232D52E}"/>
+    <hyperlink ref="H101" r:id="rId77" xr:uid="{BBB7AEA8-A3E7-2540-9D64-555CF198F0AE}"/>
+    <hyperlink ref="H102" r:id="rId78" xr:uid="{31638D57-F9A1-8440-8AAA-FB7EC3275284}"/>
+    <hyperlink ref="H103" r:id="rId79" xr:uid="{4D67B34A-C716-1048-B21D-FD65FA1FC86A}"/>
+    <hyperlink ref="H104" r:id="rId80" xr:uid="{4F9974E9-281F-324B-B2B6-DB64B7988717}"/>
+    <hyperlink ref="H105" r:id="rId81" xr:uid="{790876C7-43B0-1641-9648-4DA5B66C4E6A}"/>
+    <hyperlink ref="H106" r:id="rId82" xr:uid="{D645509F-DAD4-1B48-AE27-1756FF478CC6}"/>
+    <hyperlink ref="H107" r:id="rId83" xr:uid="{329E350C-1CF8-5C45-95C6-4C3E372F91C2}"/>
+    <hyperlink ref="H108" r:id="rId84" xr:uid="{469EFC21-E4CF-EA44-97D3-E3BC30FBA948}"/>
+    <hyperlink ref="H109" r:id="rId85" xr:uid="{6F4FFC68-88CD-BF45-B17F-2DF461BC021E}"/>
+    <hyperlink ref="H110" r:id="rId86" xr:uid="{234BD536-ADCB-C642-AC40-BC68C8BC75ED}"/>
+    <hyperlink ref="H111" r:id="rId87" xr:uid="{0F913E7E-15FD-6443-9176-9E98916E93F7}"/>
+    <hyperlink ref="H94" r:id="rId88" xr:uid="{02E7DD7A-B547-6244-A2A1-E756539494E9}"/>
+    <hyperlink ref="H95" r:id="rId89" xr:uid="{14B32940-312C-6B49-98C8-25110195771A}"/>
+    <hyperlink ref="H99" r:id="rId90" xr:uid="{FB8A849A-02BC-804A-B3EF-635EB1A65166}"/>
+    <hyperlink ref="H92" r:id="rId91" xr:uid="{65A68C2D-B57A-9B49-95D7-A2B95A5E4A2B}"/>
+    <hyperlink ref="H80" r:id="rId92" xr:uid="{67990DD2-B01E-3C4F-8FDD-D08E451508D9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>